<commit_message>
Apply latest metal collection order
</commit_message>
<xml_diff>
--- a/2026年度物件表_KMN置換.xlsx
+++ b/2026年度物件表_KMN置換.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026年度担当者物件表  20260127" sheetId="1" r:id="Rcaa4741ae488472b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日金属（行ってるとこコバ）" sheetId="2" r:id="R2eeb60777d2b4645"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日金属収集表  (改定)" sheetId="3" r:id="R7e94b7f22a304238"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日金属収集表  (uejii)" sheetId="4" r:id="R7a47181b173b48ab"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日金属収集表 " sheetId="5" r:id="Rc80b750430494b35"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日可燃収集表 (20250709)" sheetId="6" r:id="R1aaef19a2e9047d7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="土曜日物件表 20250624" sheetId="7" r:id="Rc50e6944875c46c4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ガラ集物件（20250709）" sheetId="8" r:id="R83755af76b134a66"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="非表示物件" sheetId="9" r:id="R4d76699beba34448"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="土曜日許可物件表（休出用）" sheetId="10" r:id="R561e3969b3db416b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026年度担当者物件表  20260127" sheetId="1" r:id="Rc86b62a2fcb34c2f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日金属（行ってるとこコバ）" sheetId="2" r:id="R361f6452d9c84f51"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日金属収集表  (改定)" sheetId="3" r:id="R137b68ba1416446a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日金属収集表  (uejii)" sheetId="4" r:id="Rc5967cec631b4a2c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日金属収集表 " sheetId="5" r:id="R15b896d21d664328"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日可燃収集表 (20250709)" sheetId="6" r:id="R01c8bd1b423b458a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="土曜日物件表 20250624" sheetId="7" r:id="Rf22f1124dc794c22"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ガラ集物件（20250709）" sheetId="8" r:id="Rdcf5d705750c44ca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="非表示物件" sheetId="9" r:id="R9b9d9d6ade6a41d1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="土曜日許可物件表（休出用）" sheetId="10" r:id="R22c3f8e6a7fb491d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4790,7 +4790,7 @@
         <x:v>26</x:v>
       </x:c>
       <x:c r="O57" t="str">
-        <x:v>金属-21</x:v>
+        <x:v>金属-22</x:v>
       </x:c>
       <x:c r="U57" t="s">
         <x:v>159</x:v>
@@ -4848,7 +4848,7 @@
         <x:v>38</x:v>
       </x:c>
       <x:c r="O59" t="str">
-        <x:v>金属-22</x:v>
+        <x:v>金属-21</x:v>
       </x:c>
       <x:c r="U59" t="s">
         <x:v>159</x:v>

</xml_diff>

<commit_message>
Add Koda Heights to metal collection order
</commit_message>
<xml_diff>
--- a/2026年度物件表_KMN置換.xlsx
+++ b/2026年度物件表_KMN置換.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026年度担当者物件表  20260127" sheetId="1" r:id="Rc86b62a2fcb34c2f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日金属（行ってるとこコバ）" sheetId="2" r:id="R361f6452d9c84f51"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日金属収集表  (改定)" sheetId="3" r:id="R137b68ba1416446a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日金属収集表  (uejii)" sheetId="4" r:id="Rc5967cec631b4a2c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日金属収集表 " sheetId="5" r:id="R15b896d21d664328"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日可燃収集表 (20250709)" sheetId="6" r:id="R01c8bd1b423b458a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="土曜日物件表 20250624" sheetId="7" r:id="Rf22f1124dc794c22"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ガラ集物件（20250709）" sheetId="8" r:id="Rdcf5d705750c44ca"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="非表示物件" sheetId="9" r:id="R9b9d9d6ade6a41d1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="土曜日許可物件表（休出用）" sheetId="10" r:id="R22c3f8e6a7fb491d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026年度担当者物件表  20260127" sheetId="1" r:id="R9183b7e1f6214320"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日金属（行ってるとこコバ）" sheetId="2" r:id="R887b9c07c16b4913"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日金属収集表  (改定)" sheetId="3" r:id="Rc654317f894d4cb2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日金属収集表  (uejii)" sheetId="4" r:id="Re8e4230114304a7e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日金属収集表 " sheetId="5" r:id="R764e9a3db4f24e8c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日可燃収集表 (20250709)" sheetId="6" r:id="Rfc09a234cb604ad6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="土曜日物件表 20250624" sheetId="7" r:id="R7ea0794d42054c0d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ガラ集物件（20250709）" sheetId="8" r:id="Ra32891c8a4c34765"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="非表示物件" sheetId="9" r:id="R217ace66ef324c4f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="土曜日許可物件表（休出用）" sheetId="10" r:id="R574c131254424145"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -6554,6 +6554,9 @@
       <x:c r="L116" t="s">
         <x:v>104</x:v>
       </x:c>
+      <x:c r="O116" t="str">
+        <x:v>金属-35</x:v>
+      </x:c>
     </x:row>
     <x:row r="117" ht="21" customHeight="1">
       <x:c r="A117" t="s">
@@ -6677,7 +6680,7 @@
         <x:v>130</x:v>
       </x:c>
       <x:c r="O121" t="str">
-        <x:v>金属-35</x:v>
+        <x:v>金属-36</x:v>
       </x:c>
     </x:row>
     <x:row r="122" ht="21" customHeight="1">
@@ -6813,7 +6816,7 @@
         <x:v>144</x:v>
       </x:c>
       <x:c r="O126" t="str">
-        <x:v>金属-36</x:v>
+        <x:v>金属-37</x:v>
       </x:c>
       <x:c r="Q126" t="str">
         <x:v>ガラ-</x:v>
@@ -6917,7 +6920,7 @@
         <x:v>321</x:v>
       </x:c>
       <x:c r="O130" t="str">
-        <x:v>金属-37</x:v>
+        <x:v>金属-38</x:v>
       </x:c>
       <x:c r="S130" t="s">
         <x:v>191</x:v>
@@ -7065,7 +7068,7 @@
         <x:v>40</x:v>
       </x:c>
       <x:c r="O135" t="str">
-        <x:v>金属-38</x:v>
+        <x:v>金属-39</x:v>
       </x:c>
       <x:c r="P135" t="s">
         <x:v>29</x:v>
@@ -7221,7 +7224,7 @@
         <x:v>290</x:v>
       </x:c>
       <x:c r="O141" t="str">
-        <x:v>金属-39</x:v>
+        <x:v>金属-40</x:v>
       </x:c>
     </x:row>
     <x:row r="142" ht="21" customHeight="1">
@@ -7303,7 +7306,7 @@
         <x:v>361</x:v>
       </x:c>
       <x:c r="O144" t="str">
-        <x:v>金属-40</x:v>
+        <x:v>金属-41</x:v>
       </x:c>
       <x:c r="U144" t="s">
         <x:v>126</x:v>
@@ -7335,7 +7338,7 @@
         <x:v>364</x:v>
       </x:c>
       <x:c r="O145" t="str">
-        <x:v>金属-41</x:v>
+        <x:v>金属-42</x:v>
       </x:c>
     </x:row>
     <x:row r="146" ht="21" customHeight="1">
@@ -7436,7 +7439,7 @@
         <x:v>373</x:v>
       </x:c>
       <x:c r="O149" t="str">
-        <x:v>金属-42</x:v>
+        <x:v>金属-43</x:v>
       </x:c>
     </x:row>
     <x:row r="150" ht="21" customHeight="1">
@@ -7647,7 +7650,7 @@
         <x:v>388</x:v>
       </x:c>
       <x:c r="O157" t="str">
-        <x:v>金属-43</x:v>
+        <x:v>金属-44</x:v>
       </x:c>
       <x:c r="Q157" t="str">
         <x:v>ガラ-</x:v>
@@ -7734,7 +7737,7 @@
         <x:v>346</x:v>
       </x:c>
       <x:c r="O160" t="str">
-        <x:v>金属-44</x:v>
+        <x:v>金属-45</x:v>
       </x:c>
     </x:row>
     <x:row r="161" ht="21" customHeight="1">
@@ -7775,7 +7778,7 @@
         <x:v>398</x:v>
       </x:c>
       <x:c r="O161" t="str">
-        <x:v>金属-45</x:v>
+        <x:v>金属-46</x:v>
       </x:c>
       <x:c r="P161" t="s">
         <x:v>29</x:v>
@@ -7879,7 +7882,7 @@
         <x:v>408</x:v>
       </x:c>
       <x:c r="O165" t="str">
-        <x:v>金属-46</x:v>
+        <x:v>金属-47</x:v>
       </x:c>
       <x:c r="Q165" t="str">
         <x:v>ガラ-</x:v>
@@ -8102,7 +8105,7 @@
         <x:v>373</x:v>
       </x:c>
       <x:c r="O174" t="str">
-        <x:v>金属-48</x:v>
+        <x:v>金属-49</x:v>
       </x:c>
     </x:row>
     <x:row r="175" ht="21" customHeight="1">
@@ -8189,7 +8192,7 @@
         <x:v>398</x:v>
       </x:c>
       <x:c r="O177" t="str">
-        <x:v>金属-47</x:v>
+        <x:v>金属-48</x:v>
       </x:c>
       <x:c r="Q177" t="str">
         <x:v>ガラ-</x:v>
@@ -8310,7 +8313,7 @@
         <x:v>395</x:v>
       </x:c>
       <x:c r="O182" t="str">
-        <x:v>金属-49</x:v>
+        <x:v>金属-50</x:v>
       </x:c>
     </x:row>
     <x:row r="183" ht="21" customHeight="1">
@@ -8336,7 +8339,7 @@
         <x:v>388</x:v>
       </x:c>
       <x:c r="O183" t="str">
-        <x:v>金属-50</x:v>
+        <x:v>金属-51</x:v>
       </x:c>
     </x:row>
     <x:row r="184" ht="21" customHeight="1">
@@ -8359,7 +8362,7 @@
         <x:v>38</x:v>
       </x:c>
       <x:c r="O184" t="str">
-        <x:v>金属-51</x:v>
+        <x:v>金属-52</x:v>
       </x:c>
     </x:row>
     <x:row r="185" ht="21" customHeight="1">
@@ -9440,7 +9443,7 @@
         <x:v>37</x:v>
       </x:c>
       <x:c r="O226" t="str">
-        <x:v>金属-60</x:v>
+        <x:v>金属-61</x:v>
       </x:c>
       <x:c r="Q226" t="str">
         <x:v>ガラ-</x:v>
@@ -9521,7 +9524,7 @@
         <x:v>37</x:v>
       </x:c>
       <x:c r="O229" t="str">
-        <x:v>金属-59</x:v>
+        <x:v>金属-60</x:v>
       </x:c>
       <x:c r="Q229" t="str">
         <x:v>ガラ-</x:v>
@@ -9568,7 +9571,7 @@
         <x:v>398</x:v>
       </x:c>
       <x:c r="O230" t="str">
-        <x:v>金属-58</x:v>
+        <x:v>金属-59</x:v>
       </x:c>
       <x:c r="Q230" t="str">
         <x:v>ガラ-</x:v>
@@ -9594,7 +9597,7 @@
         <x:v>37</x:v>
       </x:c>
       <x:c r="O231" t="str">
-        <x:v>金属-61</x:v>
+        <x:v>金属-62</x:v>
       </x:c>
       <x:c r="S231" t="s">
         <x:v>550</x:v>
@@ -9678,7 +9681,7 @@
         <x:v>558</x:v>
       </x:c>
       <x:c r="O234" t="str">
-        <x:v>金属-54</x:v>
+        <x:v>金属-55</x:v>
       </x:c>
     </x:row>
     <x:row r="235" ht="21" customHeight="1">
@@ -9730,7 +9733,7 @@
         <x:v>561</x:v>
       </x:c>
       <x:c r="O236" t="str">
-        <x:v>金属-56</x:v>
+        <x:v>金属-57</x:v>
       </x:c>
       <x:c r="Q236" t="str">
         <x:v>ガラ-</x:v>
@@ -9762,7 +9765,7 @@
         <x:v>564</x:v>
       </x:c>
       <x:c r="O237" t="str">
-        <x:v>金属-57</x:v>
+        <x:v>金属-58</x:v>
       </x:c>
       <x:c r="Q237" t="str">
         <x:v>ガラ-</x:v>
@@ -9791,7 +9794,7 @@
         <x:v>566</x:v>
       </x:c>
       <x:c r="O238" t="str">
-        <x:v>金属-55</x:v>
+        <x:v>金属-56</x:v>
       </x:c>
       <x:c r="Q238" t="str">
         <x:v>ガラ-</x:v>
@@ -9843,7 +9846,7 @@
         <x:v>571</x:v>
       </x:c>
       <x:c r="O240" t="str">
-        <x:v>金属-53</x:v>
+        <x:v>金属-54</x:v>
       </x:c>
       <x:c r="U240" t="s">
         <x:v>126</x:v>
@@ -9872,7 +9875,7 @@
         <x:v>574</x:v>
       </x:c>
       <x:c r="O241" t="str">
-        <x:v>金属-52</x:v>
+        <x:v>金属-53</x:v>
       </x:c>
       <x:c r="U241" t="s">
         <x:v>126</x:v>

</xml_diff>

<commit_message>
Rename main property sheet
</commit_message>
<xml_diff>
--- a/2026年度物件表_KMN置換.xlsx
+++ b/2026年度物件表_KMN置換.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026年度担当者物件表  20260127" sheetId="1" r:id="R9183b7e1f6214320"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日金属（行ってるとこコバ）" sheetId="2" r:id="R887b9c07c16b4913"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日金属収集表  (改定)" sheetId="3" r:id="Rc654317f894d4cb2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日金属収集表  (uejii)" sheetId="4" r:id="Re8e4230114304a7e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日金属収集表 " sheetId="5" r:id="R764e9a3db4f24e8c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日可燃収集表 (20250709)" sheetId="6" r:id="Rfc09a234cb604ad6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="土曜日物件表 20250624" sheetId="7" r:id="R7ea0794d42054c0d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ガラ集物件（20250709）" sheetId="8" r:id="Ra32891c8a4c34765"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="非表示物件" sheetId="9" r:id="R217ace66ef324c4f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="土曜日許可物件表（休出用）" sheetId="10" r:id="R574c131254424145"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="物件表" sheetId="1" r:id="R7f93a872f6004df7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日金属（行ってるとこコバ）" sheetId="2" r:id="R60068292d8de46f3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日金属収集表  (改定)" sheetId="3" r:id="Rb0eec0e3bc074804"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日金属収集表  (uejii)" sheetId="4" r:id="R3ecc766f70744b45"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日金属収集表 " sheetId="5" r:id="Rf997c94c31834f16"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日可燃収集表 (20250709)" sheetId="6" r:id="Re984608b9ff340bf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="土曜日物件表 20250624" sheetId="7" r:id="R42d6e6f78aa04fbd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ガラ集物件（20250709）" sheetId="8" r:id="R4183e187a90b45d7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="非表示物件" sheetId="9" r:id="R61e047fbc2524744"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="土曜日許可物件表（休出用）" sheetId="10" r:id="Rdad1a8268b8a4e2d"/>
   </x:sheets>
 </x:workbook>
 </file>

</xml_diff>

<commit_message>
Shorten Saturday route labels
</commit_message>
<xml_diff>
--- a/2026年度物件表_KMN置換.xlsx
+++ b/2026年度物件表_KMN置換.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="物件表" sheetId="1" r:id="Raf15cb858f8c47d8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日金属（行ってるとこコバ）" sheetId="2" r:id="Re3a41c346eb74efe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日金属収集表  (改定)" sheetId="3" r:id="R8cf8e9aff4f440ee"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日金属収集表  (uejii)" sheetId="4" r:id="R18751522507d4df8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日金属収集表 " sheetId="5" r:id="Re2ca50566047406c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日可燃収集表 (20250709)" sheetId="6" r:id="R2b125c5fb2d34da1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="土曜日物件表 20250624" sheetId="7" r:id="Reb968eff5ee74db6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ガラ集物件（20250709）" sheetId="8" r:id="Ra81c548538bf4a41"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="非表示物件" sheetId="9" r:id="R4ef68c06ecd84028"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="土曜日許可物件表（休出用）" sheetId="10" r:id="R676808eb10784a22"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="物件表" sheetId="1" r:id="R98982c6b66e74bb5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日金属（行ってるとこコバ）" sheetId="2" r:id="Rf9cbba4c572746be"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日金属収集表  (改定)" sheetId="3" r:id="R4f7273046b7e4ef5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日金属収集表  (uejii)" sheetId="4" r:id="R5ad7395704a348f2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日金属収集表 " sheetId="5" r:id="R6d9d6e02d9c04179"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日可燃収集表 (20250709)" sheetId="6" r:id="R28663c0829ac413d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="土曜日物件表 20250624" sheetId="7" r:id="Rec4822fcc9b34495"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ガラ集物件（20250709）" sheetId="8" r:id="R5334129fd96d4910"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="非表示物件" sheetId="9" r:id="R703f3af5bcb44af0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="土曜日許可物件表（休出用）" sheetId="10" r:id="Rc87883188d764462"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3420,7 +3420,7 @@
         <x:v>26</x:v>
       </x:c>
       <x:c r="M7" t="str">
-        <x:v>内回り-2</x:v>
+        <x:v>内-2</x:v>
       </x:c>
       <x:c r="O7" t="str">
         <x:v>金属-1</x:v>
@@ -3470,7 +3470,7 @@
         <x:v>26</x:v>
       </x:c>
       <x:c r="M8" t="str">
-        <x:v>内回り-1</x:v>
+        <x:v>内-1</x:v>
       </x:c>
       <x:c r="O8" t="str">
         <x:v>金属-2</x:v>
@@ -4053,7 +4053,7 @@
         <x:v>26</x:v>
       </x:c>
       <x:c r="M29" t="str">
-        <x:v>内回り-3</x:v>
+        <x:v>内-3</x:v>
       </x:c>
       <x:c r="O29" t="str">
         <x:v>金属-5</x:v>
@@ -4286,7 +4286,7 @@
         <x:v>26</x:v>
       </x:c>
       <x:c r="M37" t="str">
-        <x:v>内回り-6</x:v>
+        <x:v>内-6</x:v>
       </x:c>
     </x:row>
     <x:row r="38" ht="21" customHeight="1">
@@ -4391,7 +4391,7 @@
         <x:v>M-</x:v>
       </x:c>
       <x:c r="M41" t="str">
-        <x:v>外回り-15</x:v>
+        <x:v>外-15</x:v>
       </x:c>
     </x:row>
     <x:row r="42" ht="21" customHeight="1">
@@ -4509,7 +4509,7 @@
         <x:v>26</x:v>
       </x:c>
       <x:c r="M46" t="str">
-        <x:v>内回り-7</x:v>
+        <x:v>内-7</x:v>
       </x:c>
       <x:c r="O46" t="str">
         <x:v>金属-20</x:v>
@@ -5015,7 +5015,7 @@
         <x:v>26</x:v>
       </x:c>
       <x:c r="M65" t="str">
-        <x:v>内回り-8</x:v>
+        <x:v>内-8</x:v>
       </x:c>
       <x:c r="Q65" t="str">
         <x:v>ガラ-</x:v>
@@ -5299,7 +5299,7 @@
         <x:v>201</x:v>
       </x:c>
       <x:c r="M76" t="str">
-        <x:v>内回り-17</x:v>
+        <x:v>内-17</x:v>
       </x:c>
       <x:c r="S76" t="s">
         <x:v>202</x:v>
@@ -5372,7 +5372,7 @@
         <x:v>37</x:v>
       </x:c>
       <x:c r="M78" t="str">
-        <x:v>内回り-18</x:v>
+        <x:v>内-18</x:v>
       </x:c>
       <x:c r="O78" t="str"/>
     </x:row>
@@ -5486,7 +5486,7 @@
         <x:v>37</x:v>
       </x:c>
       <x:c r="M82" t="str">
-        <x:v>内回り-16</x:v>
+        <x:v>内-16</x:v>
       </x:c>
     </x:row>
     <x:row r="83" ht="21" customHeight="1">
@@ -5521,7 +5521,7 @@
         <x:v>37</x:v>
       </x:c>
       <x:c r="M83" t="str">
-        <x:v>内回り-14</x:v>
+        <x:v>内-14</x:v>
       </x:c>
     </x:row>
     <x:row r="84" ht="21" customHeight="1">
@@ -5559,7 +5559,7 @@
         <x:v>37</x:v>
       </x:c>
       <x:c r="M84" t="str">
-        <x:v>内回り-15</x:v>
+        <x:v>内-15</x:v>
       </x:c>
     </x:row>
     <x:row r="85" ht="21" customHeight="1">
@@ -5659,7 +5659,7 @@
         <x:v>37</x:v>
       </x:c>
       <x:c r="M87" t="str">
-        <x:v>内回り-13</x:v>
+        <x:v>内-13</x:v>
       </x:c>
     </x:row>
     <x:row r="88" ht="21" customHeight="1">
@@ -6074,7 +6074,7 @@
         <x:v>37</x:v>
       </x:c>
       <x:c r="M101" t="str">
-        <x:v>内回り-12</x:v>
+        <x:v>内-12</x:v>
       </x:c>
       <x:c r="O101" t="str">
         <x:v>金属-27</x:v>
@@ -6277,7 +6277,7 @@
         <x:v>37</x:v>
       </x:c>
       <x:c r="M108" t="str">
-        <x:v>外回り-14</x:v>
+        <x:v>外-14</x:v>
       </x:c>
     </x:row>
     <x:row r="109" ht="21" customHeight="1">
@@ -6318,7 +6318,7 @@
         <x:v>37</x:v>
       </x:c>
       <x:c r="M109" t="str">
-        <x:v>外回り-13</x:v>
+        <x:v>外-13</x:v>
       </x:c>
     </x:row>
     <x:row r="110" ht="21" customHeight="1">
@@ -6440,7 +6440,7 @@
         <x:v>205</x:v>
       </x:c>
       <x:c r="M113" t="str">
-        <x:v>内回り-11</x:v>
+        <x:v>内-11</x:v>
       </x:c>
       <x:c r="O113" t="str">
         <x:v>金属-33</x:v>
@@ -6963,7 +6963,7 @@
         <x:v>174</x:v>
       </x:c>
       <x:c r="M131" t="str">
-        <x:v>内回り-10</x:v>
+        <x:v>内-10</x:v>
       </x:c>
     </x:row>
     <x:row r="132" ht="21" customHeight="1">
@@ -7064,7 +7064,7 @@
         <x:v>293</x:v>
       </x:c>
       <x:c r="M135" t="str">
-        <x:v>内回り-9</x:v>
+        <x:v>内-9</x:v>
       </x:c>
       <x:c r="O135" t="str">
         <x:v>金属-39</x:v>
@@ -7577,7 +7577,7 @@
         <x:v>320</x:v>
       </x:c>
       <x:c r="M154" t="str">
-        <x:v>外回り-12</x:v>
+        <x:v>外-12</x:v>
       </x:c>
     </x:row>
     <x:row r="155" ht="21" customHeight="1">
@@ -7774,7 +7774,7 @@
         <x:v>347</x:v>
       </x:c>
       <x:c r="M161" t="str">
-        <x:v>外回り-11</x:v>
+        <x:v>外-11</x:v>
       </x:c>
       <x:c r="O161" t="str">
         <x:v>金属-46</x:v>
@@ -7973,7 +7973,7 @@
         <x:v>412</x:v>
       </x:c>
       <x:c r="M169" t="str">
-        <x:v>外回り-10</x:v>
+        <x:v>外-10</x:v>
       </x:c>
       <x:c r="U169" t="s">
         <x:v>413</x:v>
@@ -8188,7 +8188,7 @@
         <x:v>363</x:v>
       </x:c>
       <x:c r="M177" t="str">
-        <x:v>外回り-9</x:v>
+        <x:v>外-9</x:v>
       </x:c>
       <x:c r="O177" t="str">
         <x:v>金属-48</x:v>
@@ -8413,7 +8413,7 @@
         <x:v>M-</x:v>
       </x:c>
       <x:c r="M186" t="str">
-        <x:v>外回り-8</x:v>
+        <x:v>外-8</x:v>
       </x:c>
     </x:row>
     <x:row r="187" ht="21" customHeight="1">
@@ -8439,7 +8439,7 @@
         <x:v>M-</x:v>
       </x:c>
       <x:c r="M187" t="str">
-        <x:v>外回り-7</x:v>
+        <x:v>外-7</x:v>
       </x:c>
       <x:c r="U187" t="s">
         <x:v>413</x:v>
@@ -8468,7 +8468,7 @@
         <x:v>M-</x:v>
       </x:c>
       <x:c r="M188" t="str">
-        <x:v>外回り-6</x:v>
+        <x:v>外-6</x:v>
       </x:c>
     </x:row>
     <x:row r="189" ht="21" customHeight="1">
@@ -8716,7 +8716,7 @@
         <x:v>37</x:v>
       </x:c>
       <x:c r="M197" t="str">
-        <x:v>内回り-4</x:v>
+        <x:v>内-4</x:v>
       </x:c>
     </x:row>
     <x:row r="198" ht="21" customHeight="1">
@@ -8754,7 +8754,7 @@
         <x:v>37</x:v>
       </x:c>
       <x:c r="M198" t="str">
-        <x:v>内回り-5</x:v>
+        <x:v>内-5</x:v>
       </x:c>
     </x:row>
     <x:row r="199" ht="21" customHeight="1">
@@ -9567,7 +9567,7 @@
         <x:v>37</x:v>
       </x:c>
       <x:c r="M230" t="str">
-        <x:v>内回り-19</x:v>
+        <x:v>内-19</x:v>
       </x:c>
       <x:c r="O230" t="str">
         <x:v>金属-59</x:v>
@@ -10033,7 +10033,7 @@
         <x:v>26</x:v>
       </x:c>
       <x:c r="M247" t="str">
-        <x:v>外回り-5</x:v>
+        <x:v>外-5</x:v>
       </x:c>
       <x:c r="O247" t="str">
         <x:v>金属-14</x:v>
@@ -10106,7 +10106,7 @@
         <x:v>26</x:v>
       </x:c>
       <x:c r="M249" t="str">
-        <x:v>外回り-4</x:v>
+        <x:v>外-4</x:v>
       </x:c>
       <x:c r="O249" t="str">
         <x:v>金属-15</x:v>
@@ -10747,7 +10747,7 @@
         <x:v>26</x:v>
       </x:c>
       <x:c r="M274" t="str">
-        <x:v>外回り-2</x:v>
+        <x:v>外-2</x:v>
       </x:c>
       <x:c r="O274" t="str">
         <x:v>金属-7</x:v>
@@ -11033,7 +11033,7 @@
         <x:v>37</x:v>
       </x:c>
       <x:c r="M285" t="str">
-        <x:v>外回り-3</x:v>
+        <x:v>外-3</x:v>
       </x:c>
     </x:row>
     <x:row r="286" ht="21" customHeight="1">
@@ -11174,7 +11174,7 @@
         <x:v>658</x:v>
       </x:c>
       <x:c r="M291" t="str">
-        <x:v>外回り-1</x:v>
+        <x:v>外-1</x:v>
       </x:c>
     </x:row>
     <x:row r="292" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Update Kawaguchi Apartment Wednesday assignment
</commit_message>
<xml_diff>
--- a/2026年度物件表_KMN置換.xlsx
+++ b/2026年度物件表_KMN置換.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="物件表" sheetId="1" r:id="R98982c6b66e74bb5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日金属（行ってるとこコバ）" sheetId="2" r:id="Rf9cbba4c572746be"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日金属収集表  (改定)" sheetId="3" r:id="R4f7273046b7e4ef5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日金属収集表  (uejii)" sheetId="4" r:id="R5ad7395704a348f2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日金属収集表 " sheetId="5" r:id="R6d9d6e02d9c04179"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日可燃収集表 (20250709)" sheetId="6" r:id="R28663c0829ac413d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="土曜日物件表 20250624" sheetId="7" r:id="Rec4822fcc9b34495"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ガラ集物件（20250709）" sheetId="8" r:id="R5334129fd96d4910"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="非表示物件" sheetId="9" r:id="R703f3af5bcb44af0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="土曜日許可物件表（休出用）" sheetId="10" r:id="Rc87883188d764462"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="物件表" sheetId="1" r:id="R494c18ac973d424f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日金属（行ってるとこコバ）" sheetId="2" r:id="R5a6fce78678a488a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日金属収集表  (改定)" sheetId="3" r:id="R2930d3233d764956"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日金属収集表  (uejii)" sheetId="4" r:id="R052295ae13664dbc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日金属収集表 " sheetId="5" r:id="R56be17aea77241c1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日可燃収集表 (20250709)" sheetId="6" r:id="R36bac3821ff84f9d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="土曜日物件表 20250624" sheetId="7" r:id="R5c3acd7812f547d3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ガラ集物件（20250709）" sheetId="8" r:id="R84ed7a50300a4b2f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="非表示物件" sheetId="9" r:id="Rcb2c28d6fb5440f1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="土曜日許可物件表（休出用）" sheetId="10" r:id="Rcef9583c9eec46cf"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -10134,8 +10134,8 @@
       <x:c r="E250" t="s">
         <x:v>590</x:v>
       </x:c>
-      <x:c r="J250" t="s">
-        <x:v>37</x:v>
+      <x:c r="J250" t="str">
+        <x:v>M-</x:v>
       </x:c>
     </x:row>
     <x:row r="251" ht="21" customHeight="1">

</xml_diff>

<commit_message>
Add Saturday cardboard collection order
</commit_message>
<xml_diff>
--- a/2026年度物件表_KMN置換.xlsx
+++ b/2026年度物件表_KMN置換.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="物件表" sheetId="1" r:id="R494c18ac973d424f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日金属（行ってるとこコバ）" sheetId="2" r:id="R5a6fce78678a488a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日金属収集表  (改定)" sheetId="3" r:id="R2930d3233d764956"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日金属収集表  (uejii)" sheetId="4" r:id="R052295ae13664dbc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日金属収集表 " sheetId="5" r:id="R56be17aea77241c1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日可燃収集表 (20250709)" sheetId="6" r:id="R36bac3821ff84f9d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="土曜日物件表 20250624" sheetId="7" r:id="R5c3acd7812f547d3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ガラ集物件（20250709）" sheetId="8" r:id="R84ed7a50300a4b2f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="非表示物件" sheetId="9" r:id="Rcb2c28d6fb5440f1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="土曜日許可物件表（休出用）" sheetId="10" r:id="Rcef9583c9eec46cf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="物件表" sheetId="1" r:id="R1d07c582a4f24738"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日金属（行ってるとこコバ）" sheetId="2" r:id="R65479d35ecc646be"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日金属収集表  (改定)" sheetId="3" r:id="R92e3a2b1b95441db"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日金属収集表  (uejii)" sheetId="4" r:id="Rc0eac0bd21834ac4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日金属収集表 " sheetId="5" r:id="R713a1f6464024d7a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日可燃収集表 (20250709)" sheetId="6" r:id="R3a054b6a31c640cc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="土曜日物件表 20250624" sheetId="7" r:id="Re54989bc5ed8400c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ガラ集物件（20250709）" sheetId="8" r:id="R055e1a7cffa446f2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="非表示物件" sheetId="9" r:id="R003e549b51bd4f60"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="土曜日許可物件表（休出用）" sheetId="10" r:id="R63343ebc216545ef"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3510,8 +3510,8 @@
       <x:c r="L9" t="s">
         <x:v>15</x:v>
       </x:c>
-      <x:c r="M9" t="s">
-        <x:v>15</x:v>
+      <x:c r="M9" t="str">
+        <x:v>段紙(土)-10</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="21" customHeight="1">
@@ -4053,7 +4053,7 @@
         <x:v>26</x:v>
       </x:c>
       <x:c r="M29" t="str">
-        <x:v>内-3</x:v>
+        <x:v>段紙(土)-2</x:v>
       </x:c>
       <x:c r="O29" t="str">
         <x:v>金属-5</x:v>
@@ -4509,7 +4509,7 @@
         <x:v>26</x:v>
       </x:c>
       <x:c r="M46" t="str">
-        <x:v>内-7</x:v>
+        <x:v>段紙(土)-6</x:v>
       </x:c>
       <x:c r="O46" t="str">
         <x:v>金属-20</x:v>
@@ -6074,7 +6074,7 @@
         <x:v>37</x:v>
       </x:c>
       <x:c r="M101" t="str">
-        <x:v>内-12</x:v>
+        <x:v>段紙(土)-7</x:v>
       </x:c>
       <x:c r="O101" t="str">
         <x:v>金属-27</x:v>
@@ -7064,7 +7064,7 @@
         <x:v>293</x:v>
       </x:c>
       <x:c r="M135" t="str">
-        <x:v>内-9</x:v>
+        <x:v>段紙(土)-8</x:v>
       </x:c>
       <x:c r="O135" t="str">
         <x:v>金属-39</x:v>
@@ -7774,7 +7774,7 @@
         <x:v>347</x:v>
       </x:c>
       <x:c r="M161" t="str">
-        <x:v>外-11</x:v>
+        <x:v>段紙(土)-9</x:v>
       </x:c>
       <x:c r="O161" t="str">
         <x:v>金属-46</x:v>
@@ -10033,7 +10033,7 @@
         <x:v>26</x:v>
       </x:c>
       <x:c r="M247" t="str">
-        <x:v>外-5</x:v>
+        <x:v>段紙(土)-3</x:v>
       </x:c>
       <x:c r="O247" t="str">
         <x:v>金属-14</x:v>
@@ -10106,7 +10106,7 @@
         <x:v>26</x:v>
       </x:c>
       <x:c r="M249" t="str">
-        <x:v>外-4</x:v>
+        <x:v>段紙(土)-4</x:v>
       </x:c>
       <x:c r="O249" t="str">
         <x:v>金属-15</x:v>
@@ -10747,7 +10747,7 @@
         <x:v>26</x:v>
       </x:c>
       <x:c r="M274" t="str">
-        <x:v>外-2</x:v>
+        <x:v>段紙(土)-5</x:v>
       </x:c>
       <x:c r="O274" t="str">
         <x:v>金属-7</x:v>
@@ -11280,6 +11280,76 @@
       <x:c r="U295" t="s">
         <x:v>670</x:v>
       </x:c>
+    </x:row>
+    <x:row r="296">
+      <x:c r="A296" t="str">
+        <x:v>四十九</x:v>
+      </x:c>
+      <x:c r="B296" t="str">
+        <x:v>会社　商店</x:v>
+      </x:c>
+      <x:c r="C296" t="n">
+        <x:v>295</x:v>
+      </x:c>
+      <x:c r="D296" t="n">
+        <x:v>298</x:v>
+      </x:c>
+      <x:c r="E296" t="str">
+        <x:v>会社の段ボール</x:v>
+      </x:c>
+      <x:c r="F296"/>
+      <x:c r="G296"/>
+      <x:c r="H296"/>
+      <x:c r="I296"/>
+      <x:c r="J296"/>
+      <x:c r="K296"/>
+      <x:c r="L296"/>
+      <x:c r="M296" t="str">
+        <x:v>段紙(土)-1</x:v>
+      </x:c>
+      <x:c r="N296"/>
+      <x:c r="O296"/>
+      <x:c r="P296"/>
+      <x:c r="Q296"/>
+      <x:c r="R296"/>
+      <x:c r="S296"/>
+      <x:c r="T296"/>
+      <x:c r="U296"/>
+    </x:row>
+    <x:row r="297">
+      <x:c r="A297" t="str">
+        <x:v>四十九</x:v>
+      </x:c>
+      <x:c r="B297" t="str">
+        <x:v>飲食　食品</x:v>
+      </x:c>
+      <x:c r="C297" t="n">
+        <x:v>296</x:v>
+      </x:c>
+      <x:c r="D297" t="n">
+        <x:v>299</x:v>
+      </x:c>
+      <x:c r="E297" t="str">
+        <x:v>イオン PET・アルミ</x:v>
+      </x:c>
+      <x:c r="F297"/>
+      <x:c r="G297"/>
+      <x:c r="H297"/>
+      <x:c r="I297"/>
+      <x:c r="J297"/>
+      <x:c r="K297"/>
+      <x:c r="L297"/>
+      <x:c r="M297" t="str">
+        <x:v>段紙(土)-11</x:v>
+      </x:c>
+      <x:c r="N297"/>
+      <x:c r="O297"/>
+      <x:c r="P297"/>
+      <x:c r="Q297"/>
+      <x:c r="R297"/>
+      <x:c r="S297"/>
+      <x:c r="T297"/>
+      <x:c r="U297"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Move paper assignment to MaxValu
</commit_message>
<xml_diff>
--- a/2026年度物件表_KMN置換.xlsx
+++ b/2026年度物件表_KMN置換.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="物件表" sheetId="1" r:id="R09bdfd6011df473a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日金属（行ってるとこコバ）" sheetId="2" r:id="Rbbec8b3cd0584f2e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日金属収集表  (改定)" sheetId="3" r:id="R5b6e47a685534e54"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日金属収集表  (uejii)" sheetId="4" r:id="Raa8f7a66d05442c7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日金属収集表 " sheetId="5" r:id="R1918551919394c0a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日可燃収集表 (20250709)" sheetId="6" r:id="Rd251b1a586ce48cc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="土曜日物件表 20250624" sheetId="7" r:id="R8357e9ebbcb9481e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ガラ集物件（20250709）" sheetId="8" r:id="R3d5a5f4bad5d4681"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="非表示物件" sheetId="9" r:id="R9158d87bae48495d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="土曜日許可物件表（休出用）" sheetId="10" r:id="Rd522b4031dfa4a5c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="物件表" sheetId="1" r:id="R93820576eda44661"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日金属（行ってるとこコバ）" sheetId="2" r:id="R0d1471c88b514c1f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日金属収集表  (改定)" sheetId="3" r:id="Rb0510d1aab6b4c72"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日金属収集表  (uejii)" sheetId="4" r:id="R8926dd20148546d3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日金属収集表 " sheetId="5" r:id="R5c4807a355e04947"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日可燃収集表 (20250709)" sheetId="6" r:id="R733a292d769949b5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="土曜日物件表 20250624" sheetId="7" r:id="R0048c7950e164603"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ガラ集物件（20250709）" sheetId="8" r:id="R964ad6d478f443b2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="非表示物件" sheetId="9" r:id="R69bf6a779acc4145"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="土曜日許可物件表（休出用）" sheetId="10" r:id="Rc80af685f2024f0f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3616,7 +3616,9 @@
       <x:c r="N10"/>
       <x:c r="O10"/>
       <x:c r="P10"/>
-      <x:c r="Q10"/>
+      <x:c r="Q10" t="str">
+        <x:v>段紙-</x:v>
+      </x:c>
       <x:c r="R10"/>
       <x:c r="S10"/>
       <x:c r="T10"/>

</xml_diff>

<commit_message>
Apply latest property table emails
</commit_message>
<xml_diff>
--- a/2026年度物件表_KMN置換.xlsx
+++ b/2026年度物件表_KMN置換.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="物件表" sheetId="1" r:id="R1ebe07936aa54058"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日金属（行ってるとこコバ）" sheetId="2" r:id="R9f355aa890144ae0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日金属収集表  (改定)" sheetId="3" r:id="Rdcbad7f4bb7044c6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日金属収集表  (uejii)" sheetId="4" r:id="Rf6c3a6095fcf4f09"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日金属収集表 " sheetId="5" r:id="R69b256997ea04d7d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日可燃収集表 (20250709)" sheetId="6" r:id="Rf777381400084ad9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="土曜日物件表 20250624" sheetId="7" r:id="Re3612705d8924982"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ガラ集物件（20250709）" sheetId="8" r:id="R1563a90e6a7546b1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="非表示物件" sheetId="9" r:id="R40230da970b64ca5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="土曜日許可物件表（休出用）" sheetId="10" r:id="R35b563b18dc44fc2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="物件表" sheetId="1" r:id="Rc17de185a5a1410b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日金属（行ってるとこコバ）" sheetId="2" r:id="R709be1715feb4c49"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日金属収集表  (改定)" sheetId="3" r:id="Ra8e1bdaed46b4271"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日金属収集表  (uejii)" sheetId="4" r:id="Rfe883c74167b4678"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日金属収集表 " sheetId="5" r:id="R685791f530c94902"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日可燃収集表 (20250709)" sheetId="6" r:id="R24ba7273569c4285"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="土曜日物件表 20250624" sheetId="7" r:id="R2c39fb8aab694a59"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ガラ集物件（20250709）" sheetId="8" r:id="R7bb5a1bd9f624151"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="非表示物件" sheetId="9" r:id="Rdebfabcf197e4ff0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="土曜日許可物件表（休出用）" sheetId="10" r:id="R7bc802b2795a4f29"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -127,85 +127,85 @@
     <x:t xml:space="preserve">スターバックスコーヒー</x:t>
   </x:si>
   <x:si>
+    <x:t xml:space="preserve">イオンタウン可燃</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">26-7888</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">段紙・PET</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">マックスバリュ可燃</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">22-1555</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">段紙・PET・アルミ・牛乳P</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">イオンタウン段紙</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">マックス段紙</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">マックスPETアルミ紙P</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">PET アルミ</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">マックス発泡</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">発泡</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">WE CARS</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">22-8833</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">会社　商店</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">関東電化ファインテック</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">マンション</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">フォーティーナイン</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">違反ゴミのみ</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">第1第3水曜日</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">介護</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">みんなの家</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">26-4165</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">なごみの家</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">H-2</x:t>
+  </x:si>
+  <x:si>
+    <x:t xml:space="preserve">ジャルディーノブリリオ（大和リビング）</x:t>
+  </x:si>
+  <x:si>
     <x:t xml:space="preserve">K-</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">イオンタウン可燃</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">26-7888</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">段紙・PET</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">マックスバリュ可燃</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">22-1555</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">段紙・PET・アルミ・牛乳P</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">イオンタウン段紙</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">マックス段紙</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">マックスPETアルミ紙P</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">PET アルミ</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">マックス発泡</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">発泡</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">WE CARS</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">22-8833</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">会社　商店</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">関東電化ファインテック</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">マンション</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">フォーティーナイン</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">違反ゴミのみ</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">第1第3水曜日</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">介護</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">みんなの家</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">26-4165</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">なごみの家</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">H-2</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">ジャルディーノブリリオ（大和リビング）</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">金属第4水曜日</x:t>
@@ -3275,8 +3275,8 @@
       <x:c r="H6" t="str">
         <x:v>K-1</x:v>
       </x:c>
-      <x:c r="I6" t="s">
-        <x:v>36</x:v>
+      <x:c r="I6" t="str">
+        <x:v>K-1</x:v>
       </x:c>
       <x:c r="J6" t="str">
         <x:v>M-</x:v>
@@ -3312,19 +3312,19 @@
         <x:v>6</x:v>
       </x:c>
       <x:c r="E7" t="s">
+        <x:v>36</x:v>
+      </x:c>
+      <x:c r="F7" t="s">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="G7" t="s">
         <x:v>37</x:v>
-      </x:c>
-      <x:c r="F7" t="s">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="G7" t="s">
-        <x:v>38</x:v>
       </x:c>
       <x:c r="H7" t="str">
         <x:v>K-2</x:v>
       </x:c>
-      <x:c r="I7" t="s">
-        <x:v>36</x:v>
+      <x:c r="I7" t="str">
+        <x:v>K-2</x:v>
       </x:c>
       <x:c r="J7" t="str">
         <x:v>M-</x:v>
@@ -3349,7 +3349,7 @@
       </x:c>
       <x:c r="S7"/>
       <x:c r="T7" t="s">
-        <x:v>39</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="U7"/>
       <x:c r="V7"/>
@@ -3368,19 +3368,19 @@
         <x:v>7</x:v>
       </x:c>
       <x:c r="E8" t="s">
+        <x:v>39</x:v>
+      </x:c>
+      <x:c r="F8" t="s">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="G8" t="s">
         <x:v>40</x:v>
-      </x:c>
-      <x:c r="F8" t="s">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="G8" t="s">
-        <x:v>41</x:v>
       </x:c>
       <x:c r="H8" t="str">
         <x:v>K-3</x:v>
       </x:c>
-      <x:c r="I8" t="s">
-        <x:v>36</x:v>
+      <x:c r="I8" t="str">
+        <x:v>K-3</x:v>
       </x:c>
       <x:c r="J8" t="str">
         <x:v>M-</x:v>
@@ -3405,7 +3405,7 @@
       </x:c>
       <x:c r="S8"/>
       <x:c r="T8" t="s">
-        <x:v>42</x:v>
+        <x:v>41</x:v>
       </x:c>
       <x:c r="U8"/>
       <x:c r="V8"/>
@@ -3424,7 +3424,7 @@
         <x:v>8</x:v>
       </x:c>
       <x:c r="E9" t="s">
-        <x:v>43</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="F9" t="s">
         <x:v>5</x:v>
@@ -3467,7 +3467,7 @@
         <x:v>9</x:v>
       </x:c>
       <x:c r="E10" t="s">
-        <x:v>44</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="F10" t="s">
         <x:v>5</x:v>
@@ -3510,22 +3510,22 @@
         <x:v>10</x:v>
       </x:c>
       <x:c r="E11" t="s">
+        <x:v>44</x:v>
+      </x:c>
+      <x:c r="F11" t="s">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="H11" t="s">
         <x:v>45</x:v>
       </x:c>
-      <x:c r="F11" t="s">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="H11" t="s">
-        <x:v>46</x:v>
-      </x:c>
       <x:c r="J11" t="s">
-        <x:v>46</x:v>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="L11" t="s">
-        <x:v>46</x:v>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="M11" t="s">
-        <x:v>46</x:v>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="N11"/>
       <x:c r="O11"/>
@@ -3551,19 +3551,19 @@
         <x:v>11</x:v>
       </x:c>
       <x:c r="E12" t="s">
+        <x:v>46</x:v>
+      </x:c>
+      <x:c r="F12" t="s">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="H12" t="s">
         <x:v>47</x:v>
       </x:c>
-      <x:c r="F12" t="s">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="H12" t="s">
-        <x:v>48</x:v>
-      </x:c>
       <x:c r="J12" t="s">
-        <x:v>48</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="L12" t="s">
-        <x:v>48</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="N12"/>
       <x:c r="O12"/>
@@ -3589,16 +3589,16 @@
         <x:v>12</x:v>
       </x:c>
       <x:c r="E13" t="s">
+        <x:v>48</x:v>
+      </x:c>
+      <x:c r="G13" t="s">
         <x:v>49</x:v>
-      </x:c>
-      <x:c r="G13" t="s">
-        <x:v>50</x:v>
       </x:c>
       <x:c r="H13" t="str">
         <x:v>K-4</x:v>
       </x:c>
-      <x:c r="I13" t="s">
-        <x:v>36</x:v>
+      <x:c r="I13" t="str">
+        <x:v>K-4</x:v>
       </x:c>
       <x:c r="J13" t="str">
         <x:v>M-</x:v>
@@ -3626,7 +3626,7 @@
         <x:v>21</x:v>
       </x:c>
       <x:c r="B14" t="s">
-        <x:v>51</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C14">
         <x:v>13</x:v>
@@ -3635,7 +3635,7 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="E14" t="s">
-        <x:v>52</x:v>
+        <x:v>51</x:v>
       </x:c>
       <x:c r="L14" t="s">
         <x:v>26</x:v>
@@ -3655,7 +3655,7 @@
         <x:v>21</x:v>
       </x:c>
       <x:c r="B15" t="s">
-        <x:v>53</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="C15">
         <x:v>14</x:v>
@@ -3664,7 +3664,7 @@
         <x:v>14</x:v>
       </x:c>
       <x:c r="E15" t="s">
-        <x:v>54</x:v>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="J15" t="str">
         <x:v>M-</x:v>
@@ -3678,11 +3678,11 @@
       <x:c r="R15"/>
       <x:c r="S15"/>
       <x:c r="T15" t="s">
-        <x:v>55</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="U15"/>
       <x:c r="V15" t="s">
-        <x:v>56</x:v>
+        <x:v>55</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="21" customHeight="1">
@@ -3690,7 +3690,7 @@
         <x:v>21</x:v>
       </x:c>
       <x:c r="B16" t="s">
-        <x:v>57</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="C16">
         <x:v>15</x:v>
@@ -3699,13 +3699,13 @@
         <x:v>15</x:v>
       </x:c>
       <x:c r="E16" t="s">
+        <x:v>57</x:v>
+      </x:c>
+      <x:c r="G16" t="s">
         <x:v>58</x:v>
       </x:c>
-      <x:c r="G16" t="s">
-        <x:v>59</x:v>
-      </x:c>
-      <x:c r="I16" t="s">
-        <x:v>36</x:v>
+      <x:c r="I16" t="str">
+        <x:v>K-7</x:v>
       </x:c>
       <x:c r="L16" t="s">
         <x:v>26</x:v>
@@ -3725,7 +3725,7 @@
         <x:v>21</x:v>
       </x:c>
       <x:c r="B17" t="s">
-        <x:v>57</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="C17">
         <x:v>16</x:v>
@@ -3734,10 +3734,10 @@
         <x:v>16</x:v>
       </x:c>
       <x:c r="E17" t="s">
+        <x:v>59</x:v>
+      </x:c>
+      <x:c r="H17" t="s">
         <x:v>60</x:v>
-      </x:c>
-      <x:c r="H17" t="s">
-        <x:v>61</x:v>
       </x:c>
       <x:c r="J17" t="str">
         <x:v>K-1</x:v>
@@ -3760,7 +3760,7 @@
         <x:v>21</x:v>
       </x:c>
       <x:c r="B18" t="s">
-        <x:v>53</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="C18">
         <x:v>17</x:v>
@@ -3769,10 +3769,10 @@
         <x:v>17</x:v>
       </x:c>
       <x:c r="E18" t="s">
+        <x:v>61</x:v>
+      </x:c>
+      <x:c r="I18" t="s">
         <x:v>62</x:v>
-      </x:c>
-      <x:c r="I18" t="s">
-        <x:v>36</x:v>
       </x:c>
       <x:c r="L18" t="s">
         <x:v>26</x:v>
@@ -3805,8 +3805,8 @@
       <x:c r="E19" t="s">
         <x:v>64</x:v>
       </x:c>
-      <x:c r="I19" t="s">
-        <x:v>36</x:v>
+      <x:c r="I19" t="str">
+        <x:v>K-5</x:v>
       </x:c>
       <x:c r="L19" t="s">
         <x:v>26</x:v>
@@ -3826,7 +3826,7 @@
         <x:v>21</x:v>
       </x:c>
       <x:c r="B20" t="s">
-        <x:v>57</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="C20">
         <x:v>19</x:v>
@@ -3837,8 +3837,8 @@
       <x:c r="E20" t="s">
         <x:v>65</x:v>
       </x:c>
-      <x:c r="I20" t="s">
-        <x:v>36</x:v>
+      <x:c r="I20" t="str">
+        <x:v>K-6</x:v>
       </x:c>
       <x:c r="L20" t="str">
         <x:v>M-</x:v>
@@ -3858,7 +3858,7 @@
         <x:v>66</x:v>
       </x:c>
       <x:c r="B21" t="s">
-        <x:v>51</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C21">
         <x:v>20</x:v>
@@ -3887,7 +3887,7 @@
         <x:v>66</x:v>
       </x:c>
       <x:c r="B22" t="s">
-        <x:v>51</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C22">
         <x:v>21</x:v>
@@ -3916,7 +3916,7 @@
         <x:v>66</x:v>
       </x:c>
       <x:c r="B23" t="s">
-        <x:v>51</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C23">
         <x:v>22</x:v>
@@ -3930,8 +3930,8 @@
       <x:c r="G23" t="s">
         <x:v>71</x:v>
       </x:c>
-      <x:c r="I23" t="s">
-        <x:v>36</x:v>
+      <x:c r="I23" t="str">
+        <x:v>K-9</x:v>
       </x:c>
       <x:c r="L23" t="s">
         <x:v>26</x:v>
@@ -3955,7 +3955,7 @@
         <x:v>66</x:v>
       </x:c>
       <x:c r="B24" t="s">
-        <x:v>51</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C24">
         <x:v>23</x:v>
@@ -3989,7 +3989,7 @@
         <x:v>66</x:v>
       </x:c>
       <x:c r="B25" t="s">
-        <x:v>51</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C25">
         <x:v>24</x:v>
@@ -4035,8 +4035,8 @@
       <x:c r="G26" t="s">
         <x:v>78</x:v>
       </x:c>
-      <x:c r="I26" t="s">
-        <x:v>36</x:v>
+      <x:c r="I26" t="str">
+        <x:v>K-8</x:v>
       </x:c>
       <x:c r="L26" t="s">
         <x:v>26</x:v>
@@ -4096,7 +4096,7 @@
         <x:v>66</x:v>
       </x:c>
       <x:c r="B28" t="s">
-        <x:v>57</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="C28">
         <x:v>27</x:v>
@@ -4142,8 +4142,8 @@
       <x:c r="H29" t="s">
         <x:v>86</x:v>
       </x:c>
-      <x:c r="I29" t="s">
-        <x:v>36</x:v>
+      <x:c r="I29" t="str">
+        <x:v>K-10</x:v>
       </x:c>
       <x:c r="J29" t="str">
         <x:v>K-2</x:v>
@@ -4180,7 +4180,7 @@
         <x:v>89</x:v>
       </x:c>
       <x:c r="B30" t="s">
-        <x:v>57</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="C30">
         <x:v>29</x:v>
@@ -4209,7 +4209,7 @@
         <x:v>89</x:v>
       </x:c>
       <x:c r="B31" t="s">
-        <x:v>53</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="C31">
         <x:v>30</x:v>
@@ -4223,8 +4223,8 @@
       <x:c r="G31" t="s">
         <x:v>92</x:v>
       </x:c>
-      <x:c r="I31" t="s">
-        <x:v>36</x:v>
+      <x:c r="I31" t="str">
+        <x:v>K-11</x:v>
       </x:c>
       <x:c r="N31"/>
       <x:c r="O31"/>
@@ -4241,7 +4241,7 @@
         <x:v>89</x:v>
       </x:c>
       <x:c r="B32" t="s">
-        <x:v>53</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="C32">
         <x:v>31</x:v>
@@ -4252,9 +4252,7 @@
       <x:c r="E32" t="s">
         <x:v>93</x:v>
       </x:c>
-      <x:c r="I32" t="s">
-        <x:v>36</x:v>
-      </x:c>
+      <x:c r="I32"/>
       <x:c r="J32" t="str">
         <x:v>M-</x:v>
       </x:c>
@@ -4277,7 +4275,7 @@
         <x:v>89</x:v>
       </x:c>
       <x:c r="B33" t="s">
-        <x:v>53</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="C33">
         <x:v>32</x:v>
@@ -4330,8 +4328,8 @@
       <x:c r="H34" t="str">
         <x:v>K-5</x:v>
       </x:c>
-      <x:c r="I34" t="s">
-        <x:v>36</x:v>
+      <x:c r="I34" t="str">
+        <x:v>K-12</x:v>
       </x:c>
       <x:c r="J34" t="str">
         <x:v>M-</x:v>
@@ -4357,7 +4355,7 @@
         <x:v>100</x:v>
       </x:c>
       <x:c r="B35" t="s">
-        <x:v>51</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C35">
         <x:v>34</x:v>
@@ -4441,8 +4439,8 @@
       <x:c r="H37" t="str">
         <x:v>K-6</x:v>
       </x:c>
-      <x:c r="I37" t="s">
-        <x:v>36</x:v>
+      <x:c r="I37" t="str">
+        <x:v>K-14</x:v>
       </x:c>
       <x:c r="J37" t="str">
         <x:v>M-</x:v>
@@ -4503,7 +4501,7 @@
         <x:v>100</x:v>
       </x:c>
       <x:c r="B39" t="s">
-        <x:v>53</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="C39">
         <x:v>38</x:v>
@@ -4514,8 +4512,8 @@
       <x:c r="E39" t="s">
         <x:v>113</x:v>
       </x:c>
-      <x:c r="I39" t="s">
-        <x:v>36</x:v>
+      <x:c r="I39" t="str">
+        <x:v>K-15</x:v>
       </x:c>
       <x:c r="L39" t="s">
         <x:v>26</x:v>
@@ -4636,7 +4634,7 @@
         <x:v>100</x:v>
       </x:c>
       <x:c r="B43" t="s">
-        <x:v>51</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C43">
         <x:v>42</x:v>
@@ -4665,7 +4663,7 @@
         <x:v>100</x:v>
       </x:c>
       <x:c r="B44" t="s">
-        <x:v>53</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="C44">
         <x:v>43</x:v>
@@ -4740,8 +4738,8 @@
       <x:c r="H46" t="s">
         <x:v>96</x:v>
       </x:c>
-      <x:c r="I46" t="s">
-        <x:v>36</x:v>
+      <x:c r="I46" t="str">
+        <x:v>K-16</x:v>
       </x:c>
       <x:c r="J46" t="str">
         <x:v>M-</x:v>
@@ -4776,7 +4774,7 @@
         <x:v>100</x:v>
       </x:c>
       <x:c r="B47" t="s">
-        <x:v>51</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C47">
         <x:v>46</x:v>
@@ -4874,7 +4872,7 @@
         <x:v>100</x:v>
       </x:c>
       <x:c r="B50" t="s">
-        <x:v>51</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C50">
         <x:v>49</x:v>
@@ -4909,7 +4907,7 @@
         <x:v>100</x:v>
       </x:c>
       <x:c r="B51" t="s">
-        <x:v>53</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="C51">
         <x:v>50</x:v>
@@ -4941,7 +4939,7 @@
         <x:v>100</x:v>
       </x:c>
       <x:c r="B52" t="s">
-        <x:v>51</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C52">
         <x:v>51</x:v>
@@ -4979,7 +4977,7 @@
         <x:v>100</x:v>
       </x:c>
       <x:c r="B53" t="s">
-        <x:v>51</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C53">
         <x:v>52</x:v>
@@ -5027,9 +5025,10 @@
       <x:c r="G54" t="s">
         <x:v>144</x:v>
       </x:c>
-      <x:c r="I54" t="s">
-        <x:v>36</x:v>
-      </x:c>
+      <x:c r="I54" t="str">
+        <x:v>K-</x:v>
+      </x:c>
+      <x:c r="J54"/>
       <x:c r="N54"/>
       <x:c r="O54"/>
       <x:c r="P54"/>
@@ -5360,7 +5359,7 @@
         <x:v>157</x:v>
       </x:c>
       <x:c r="B64" t="s">
-        <x:v>53</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="C64">
         <x:v>63</x:v>
@@ -5409,8 +5408,8 @@
       <x:c r="H65" t="s">
         <x:v>96</x:v>
       </x:c>
-      <x:c r="I65" t="s">
-        <x:v>36</x:v>
+      <x:c r="I65" t="str">
+        <x:v>K-18</x:v>
       </x:c>
       <x:c r="J65" t="str">
         <x:v>M-</x:v>
@@ -5441,7 +5440,7 @@
         <x:v>157</x:v>
       </x:c>
       <x:c r="B66" t="s">
-        <x:v>51</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C66">
         <x:v>65</x:v>
@@ -5452,8 +5451,8 @@
       <x:c r="E66" t="s">
         <x:v>170</x:v>
       </x:c>
-      <x:c r="I66" t="s">
-        <x:v>36</x:v>
+      <x:c r="I66" t="str">
+        <x:v>K-17</x:v>
       </x:c>
       <x:c r="N66"/>
       <x:c r="O66"/>
@@ -5533,7 +5532,7 @@
         <x:v>157</x:v>
       </x:c>
       <x:c r="B69" t="s">
-        <x:v>51</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C69">
         <x:v>68</x:v>
@@ -5562,7 +5561,7 @@
         <x:v>157</x:v>
       </x:c>
       <x:c r="B70" t="s">
-        <x:v>51</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C70">
         <x:v>69</x:v>
@@ -5633,7 +5632,7 @@
         <x:v>157</x:v>
       </x:c>
       <x:c r="B72" t="s">
-        <x:v>53</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="C72">
         <x:v>71</x:v>
@@ -5711,7 +5710,7 @@
         <x:v>157</x:v>
       </x:c>
       <x:c r="B74" t="s">
-        <x:v>51</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C74">
         <x:v>73</x:v>
@@ -5967,7 +5966,7 @@
         <x:v>194</x:v>
       </x:c>
       <x:c r="B81" t="s">
-        <x:v>53</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="C81">
         <x:v>80</x:v>
@@ -6516,7 +6515,7 @@
         <x:v>229</x:v>
       </x:c>
       <x:c r="B94" t="s">
-        <x:v>57</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="C94">
         <x:v>93</x:v>
@@ -6583,7 +6582,7 @@
         <x:v>229</x:v>
       </x:c>
       <x:c r="B96" t="s">
-        <x:v>57</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="C96">
         <x:v>95</x:v>
@@ -6615,7 +6614,7 @@
         <x:v>229</x:v>
       </x:c>
       <x:c r="B97" t="s">
-        <x:v>53</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="C97">
         <x:v>96</x:v>
@@ -6647,7 +6646,7 @@
         <x:v>229</x:v>
       </x:c>
       <x:c r="B98" t="s">
-        <x:v>51</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C98">
         <x:v>97</x:v>
@@ -6805,7 +6804,7 @@
         <x:v>229</x:v>
       </x:c>
       <x:c r="B102" t="s">
-        <x:v>53</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="C102">
         <x:v>101</x:v>
@@ -6839,7 +6838,7 @@
         <x:v>229</x:v>
       </x:c>
       <x:c r="B103" t="s">
-        <x:v>53</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="C103">
         <x:v>102</x:v>
@@ -6873,7 +6872,7 @@
         <x:v>229</x:v>
       </x:c>
       <x:c r="B104" t="s">
-        <x:v>53</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="C104">
         <x:v>103</x:v>
@@ -6912,7 +6911,7 @@
         <x:v>229</x:v>
       </x:c>
       <x:c r="B105" t="s">
-        <x:v>53</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="C105">
         <x:v>104</x:v>
@@ -7013,7 +7012,7 @@
         <x:v>229</x:v>
       </x:c>
       <x:c r="B108" t="s">
-        <x:v>57</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="C108">
         <x:v>107</x:v>
@@ -7030,8 +7029,8 @@
       <x:c r="H108" t="str">
         <x:v>K-32</x:v>
       </x:c>
-      <x:c r="I108" t="s">
-        <x:v>36</x:v>
+      <x:c r="I108" t="str">
+        <x:v>K-19</x:v>
       </x:c>
       <x:c r="J108" t="str">
         <x:v>M-</x:v>
@@ -7060,7 +7059,7 @@
         <x:v>229</x:v>
       </x:c>
       <x:c r="B109" t="s">
-        <x:v>57</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="C109">
         <x:v>108</x:v>
@@ -7080,8 +7079,8 @@
       <x:c r="H109" t="str">
         <x:v>K-33</x:v>
       </x:c>
-      <x:c r="I109" t="s">
-        <x:v>36</x:v>
+      <x:c r="I109" t="str">
+        <x:v>K-20</x:v>
       </x:c>
       <x:c r="J109" t="str">
         <x:v>M-</x:v>
@@ -7184,7 +7183,7 @@
         <x:v>229</x:v>
       </x:c>
       <x:c r="B112" t="s">
-        <x:v>53</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="C112">
         <x:v>111</x:v>
@@ -7365,7 +7364,7 @@
         <x:v>265</x:v>
       </x:c>
       <x:c r="B116" t="s">
-        <x:v>53</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="C116">
         <x:v>115</x:v>
@@ -7399,7 +7398,7 @@
         <x:v>265</x:v>
       </x:c>
       <x:c r="B117" t="s">
-        <x:v>53</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="C117">
         <x:v>116</x:v>
@@ -7428,7 +7427,7 @@
         <x:v>265</x:v>
       </x:c>
       <x:c r="B118" t="s">
-        <x:v>51</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C118">
         <x:v>117</x:v>
@@ -7527,7 +7526,7 @@
         <x:v>265</x:v>
       </x:c>
       <x:c r="B121" t="s">
-        <x:v>51</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C121">
         <x:v>120</x:v>
@@ -7642,7 +7641,7 @@
         <x:v>265</x:v>
       </x:c>
       <x:c r="B124" t="s">
-        <x:v>53</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="C124">
         <x:v>123</x:v>
@@ -7674,7 +7673,7 @@
         <x:v>265</x:v>
       </x:c>
       <x:c r="B125" t="s">
-        <x:v>53</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="C125">
         <x:v>124</x:v>
@@ -7748,7 +7747,7 @@
         <x:v>265</x:v>
       </x:c>
       <x:c r="B127" t="s">
-        <x:v>53</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="C127">
         <x:v>126</x:v>
@@ -7780,7 +7779,7 @@
         <x:v>265</x:v>
       </x:c>
       <x:c r="B128" t="s">
-        <x:v>53</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="C128">
         <x:v>127</x:v>
@@ -7812,7 +7811,7 @@
         <x:v>265</x:v>
       </x:c>
       <x:c r="B129" t="s">
-        <x:v>53</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="C129">
         <x:v>128</x:v>
@@ -7846,7 +7845,7 @@
         <x:v>265</x:v>
       </x:c>
       <x:c r="B130" t="s">
-        <x:v>53</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="C130">
         <x:v>129</x:v>
@@ -7935,7 +7934,7 @@
         <x:v>265</x:v>
       </x:c>
       <x:c r="B132" t="s">
-        <x:v>53</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="C132">
         <x:v>131</x:v>
@@ -8078,7 +8077,7 @@
         <x:v>265</x:v>
       </x:c>
       <x:c r="B136" t="s">
-        <x:v>53</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="C136">
         <x:v>135</x:v>
@@ -8110,7 +8109,7 @@
         <x:v>265</x:v>
       </x:c>
       <x:c r="B137" t="s">
-        <x:v>53</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="C137">
         <x:v>136</x:v>
@@ -8145,7 +8144,7 @@
         <x:v>265</x:v>
       </x:c>
       <x:c r="B138" t="s">
-        <x:v>53</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="C138">
         <x:v>137</x:v>
@@ -8212,7 +8211,7 @@
         <x:v>265</x:v>
       </x:c>
       <x:c r="B140" t="s">
-        <x:v>53</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="C140">
         <x:v>139</x:v>
@@ -8284,7 +8283,7 @@
         <x:v>265</x:v>
       </x:c>
       <x:c r="B142" t="s">
-        <x:v>53</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="C142">
         <x:v>141</x:v>
@@ -8430,7 +8429,7 @@
         <x:v>331</x:v>
       </x:c>
       <x:c r="B146" t="s">
-        <x:v>51</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C146">
         <x:v>145</x:v>
@@ -8467,7 +8466,7 @@
         <x:v>341</x:v>
       </x:c>
       <x:c r="B147" t="s">
-        <x:v>53</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="C147">
         <x:v>146</x:v>
@@ -8499,7 +8498,7 @@
         <x:v>341</x:v>
       </x:c>
       <x:c r="B148" t="s">
-        <x:v>51</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C148">
         <x:v>147</x:v>
@@ -8528,7 +8527,7 @@
         <x:v>341</x:v>
       </x:c>
       <x:c r="B149" t="s">
-        <x:v>53</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="C149">
         <x:v>148</x:v>
@@ -8667,7 +8666,7 @@
         <x:v>341</x:v>
       </x:c>
       <x:c r="B153" t="s">
-        <x:v>53</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="C153">
         <x:v>152</x:v>
@@ -8749,7 +8748,7 @@
         <x:v>341</x:v>
       </x:c>
       <x:c r="B155" t="s">
-        <x:v>51</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C155">
         <x:v>154</x:v>
@@ -8816,7 +8815,7 @@
         <x:v>341</x:v>
       </x:c>
       <x:c r="B157" t="s">
-        <x:v>53</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="C157">
         <x:v>156</x:v>
@@ -8849,7 +8848,7 @@
         <x:v>362</x:v>
       </x:c>
       <x:c r="B158" t="s">
-        <x:v>51</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C158">
         <x:v>157</x:v>
@@ -8884,7 +8883,7 @@
         <x:v>362</x:v>
       </x:c>
       <x:c r="B159" t="s">
-        <x:v>51</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C159">
         <x:v>158</x:v>
@@ -9012,7 +9011,7 @@
         <x:v>362</x:v>
       </x:c>
       <x:c r="B162" t="s">
-        <x:v>51</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C162">
         <x:v>161</x:v>
@@ -9046,7 +9045,7 @@
         <x:v>362</x:v>
       </x:c>
       <x:c r="B163" t="s">
-        <x:v>51</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C163">
         <x:v>162</x:v>
@@ -9083,7 +9082,7 @@
         <x:v>362</x:v>
       </x:c>
       <x:c r="B164" t="s">
-        <x:v>53</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="C164">
         <x:v>163</x:v>
@@ -9112,7 +9111,7 @@
         <x:v>362</x:v>
       </x:c>
       <x:c r="B165" t="s">
-        <x:v>53</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="C165">
         <x:v>164</x:v>
@@ -9180,7 +9179,7 @@
         <x:v>362</x:v>
       </x:c>
       <x:c r="B167" t="s">
-        <x:v>53</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="C167">
         <x:v>166</x:v>
@@ -9212,7 +9211,7 @@
         <x:v>362</x:v>
       </x:c>
       <x:c r="B168" t="s">
-        <x:v>51</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C168">
         <x:v>167</x:v>
@@ -9275,7 +9274,7 @@
         <x:v>362</x:v>
       </x:c>
       <x:c r="B170" t="s">
-        <x:v>57</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="C170">
         <x:v>169</x:v>
@@ -9307,7 +9306,7 @@
         <x:v>362</x:v>
       </x:c>
       <x:c r="B171" t="s">
-        <x:v>53</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="C171">
         <x:v>170</x:v>
@@ -9339,7 +9338,7 @@
         <x:v>362</x:v>
       </x:c>
       <x:c r="B172" t="s">
-        <x:v>51</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C172">
         <x:v>171</x:v>
@@ -9371,7 +9370,7 @@
         <x:v>362</x:v>
       </x:c>
       <x:c r="B173" t="s">
-        <x:v>51</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C173">
         <x:v>172</x:v>
@@ -9446,7 +9445,7 @@
         <x:v>362</x:v>
       </x:c>
       <x:c r="B175" t="s">
-        <x:v>51</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C175">
         <x:v>174</x:v>
@@ -9475,7 +9474,7 @@
         <x:v>362</x:v>
       </x:c>
       <x:c r="B176" t="s">
-        <x:v>51</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C176">
         <x:v>175</x:v>
@@ -9561,7 +9560,7 @@
         <x:v>362</x:v>
       </x:c>
       <x:c r="B178" t="s">
-        <x:v>51</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C178">
         <x:v>177</x:v>
@@ -9590,7 +9589,7 @@
         <x:v>362</x:v>
       </x:c>
       <x:c r="B179" t="s">
-        <x:v>51</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C179">
         <x:v>178</x:v>
@@ -9660,7 +9659,7 @@
         <x:v>362</x:v>
       </x:c>
       <x:c r="B181" t="s">
-        <x:v>51</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C181">
         <x:v>180</x:v>
@@ -9689,7 +9688,7 @@
         <x:v>411</x:v>
       </x:c>
       <x:c r="B182" t="s">
-        <x:v>53</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="C182">
         <x:v>181</x:v>
@@ -9723,7 +9722,7 @@
         <x:v>411</x:v>
       </x:c>
       <x:c r="B183" t="s">
-        <x:v>53</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="C183">
         <x:v>182</x:v>
@@ -9757,7 +9756,7 @@
         <x:v>411</x:v>
       </x:c>
       <x:c r="B184" t="s">
-        <x:v>51</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C184">
         <x:v>183</x:v>
@@ -9820,7 +9819,7 @@
         <x:v>411</x:v>
       </x:c>
       <x:c r="B186" t="s">
-        <x:v>51</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C186">
         <x:v>185</x:v>
@@ -9930,7 +9929,7 @@
         <x:v>411</x:v>
       </x:c>
       <x:c r="B189" t="s">
-        <x:v>51</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C189">
         <x:v>188</x:v>
@@ -9974,7 +9973,7 @@
         <x:v>427</x:v>
       </x:c>
       <x:c r="H190" t="s">
-        <x:v>36</x:v>
+        <x:v>62</x:v>
       </x:c>
       <x:c r="J190" t="str">
         <x:v>K-26</x:v>
@@ -9999,7 +9998,7 @@
         <x:v>425</x:v>
       </x:c>
       <x:c r="B191" t="s">
-        <x:v>51</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C191">
         <x:v>190</x:v>
@@ -10017,7 +10016,7 @@
         <x:v>429</x:v>
       </x:c>
       <x:c r="H191" t="s">
-        <x:v>36</x:v>
+        <x:v>62</x:v>
       </x:c>
       <x:c r="J191" t="str">
         <x:v>K-25</x:v>
@@ -10074,7 +10073,7 @@
         <x:v>425</x:v>
       </x:c>
       <x:c r="B193" t="s">
-        <x:v>57</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="C193">
         <x:v>192</x:v>
@@ -10106,7 +10105,7 @@
         <x:v>425</x:v>
       </x:c>
       <x:c r="B194" t="s">
-        <x:v>51</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C194">
         <x:v>193</x:v>
@@ -10120,8 +10119,8 @@
       <x:c r="G194" t="s">
         <x:v>435</x:v>
       </x:c>
-      <x:c r="I194" t="s">
-        <x:v>36</x:v>
+      <x:c r="I194" t="str">
+        <x:v>K-51</x:v>
       </x:c>
       <x:c r="L194" t="str">
         <x:v>K-52</x:v>
@@ -10141,7 +10140,7 @@
         <x:v>425</x:v>
       </x:c>
       <x:c r="B195" t="s">
-        <x:v>51</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C195">
         <x:v>194</x:v>
@@ -10155,8 +10154,8 @@
       <x:c r="G195" t="s">
         <x:v>437</x:v>
       </x:c>
-      <x:c r="I195" t="s">
-        <x:v>36</x:v>
+      <x:c r="I195" t="str">
+        <x:v>K-52</x:v>
       </x:c>
       <x:c r="L195" t="str">
         <x:v>K-53</x:v>
@@ -10176,7 +10175,7 @@
         <x:v>438</x:v>
       </x:c>
       <x:c r="B196" t="s">
-        <x:v>51</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C196">
         <x:v>195</x:v>
@@ -10225,8 +10224,8 @@
       <x:c r="H197" t="str">
         <x:v>K-47</x:v>
       </x:c>
-      <x:c r="I197" t="s">
-        <x:v>36</x:v>
+      <x:c r="I197" t="str">
+        <x:v>K-54</x:v>
       </x:c>
       <x:c r="J197" t="str">
         <x:v>K-28</x:v>
@@ -10272,8 +10271,8 @@
       <x:c r="H198" t="str">
         <x:v>K-48</x:v>
       </x:c>
-      <x:c r="I198" t="s">
-        <x:v>36</x:v>
+      <x:c r="I198" t="str">
+        <x:v>K-55</x:v>
       </x:c>
       <x:c r="J198" t="str">
         <x:v>K-29</x:v>
@@ -10302,7 +10301,7 @@
         <x:v>440</x:v>
       </x:c>
       <x:c r="B199" t="s">
-        <x:v>53</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="C199">
         <x:v>198</x:v>
@@ -10375,7 +10374,7 @@
         <x:v>440</x:v>
       </x:c>
       <x:c r="B201" t="s">
-        <x:v>51</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C201">
         <x:v>200</x:v>
@@ -10407,7 +10406,7 @@
         <x:v>440</x:v>
       </x:c>
       <x:c r="B202" t="s">
-        <x:v>51</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C202">
         <x:v>201</x:v>
@@ -10436,7 +10435,7 @@
         <x:v>453</x:v>
       </x:c>
       <x:c r="B203" t="s">
-        <x:v>57</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="C203">
         <x:v>202</x:v>
@@ -10450,8 +10449,8 @@
       <x:c r="G203" t="s">
         <x:v>455</x:v>
       </x:c>
-      <x:c r="I203" t="s">
-        <x:v>36</x:v>
+      <x:c r="I203" t="str">
+        <x:v>K-53</x:v>
       </x:c>
       <x:c r="L203" t="str">
         <x:v>K-51</x:v>
@@ -10471,7 +10470,7 @@
         <x:v>456</x:v>
       </x:c>
       <x:c r="B204" t="s">
-        <x:v>51</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C204">
         <x:v>203</x:v>
@@ -10481,6 +10480,9 @@
       </x:c>
       <x:c r="E204" t="s">
         <x:v>457</x:v>
+      </x:c>
+      <x:c r="I204" t="str">
+        <x:v>K-37</x:v>
       </x:c>
       <x:c r="L204" t="str">
         <x:v>K-36</x:v>
@@ -10500,7 +10502,7 @@
         <x:v>456</x:v>
       </x:c>
       <x:c r="B205" t="s">
-        <x:v>53</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="C205">
         <x:v>204</x:v>
@@ -10537,7 +10539,7 @@
         <x:v>456</x:v>
       </x:c>
       <x:c r="B206" t="s">
-        <x:v>51</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C206">
         <x:v>205</x:v>
@@ -10575,7 +10577,7 @@
         <x:v>456</x:v>
       </x:c>
       <x:c r="B207" t="s">
-        <x:v>51</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C207">
         <x:v>206</x:v>
@@ -10592,8 +10594,8 @@
       <x:c r="G207" t="s">
         <x:v>464</x:v>
       </x:c>
-      <x:c r="I207" t="s">
-        <x:v>36</x:v>
+      <x:c r="I207" t="str">
+        <x:v>K-39</x:v>
       </x:c>
       <x:c r="L207" t="str">
         <x:v>K-38</x:v>
@@ -10613,7 +10615,7 @@
         <x:v>456</x:v>
       </x:c>
       <x:c r="B208" t="s">
-        <x:v>51</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C208">
         <x:v>207</x:v>
@@ -10642,7 +10644,7 @@
         <x:v>466</x:v>
       </x:c>
       <x:c r="B209" t="s">
-        <x:v>51</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C209">
         <x:v>208</x:v>
@@ -10656,8 +10658,8 @@
       <x:c r="F209" t="s">
         <x:v>5</x:v>
       </x:c>
-      <x:c r="I209" t="s">
-        <x:v>36</x:v>
+      <x:c r="I209" t="str">
+        <x:v>K-38</x:v>
       </x:c>
       <x:c r="L209" t="str">
         <x:v>K-37</x:v>
@@ -10677,7 +10679,7 @@
         <x:v>466</x:v>
       </x:c>
       <x:c r="B210" t="s">
-        <x:v>51</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C210">
         <x:v>209</x:v>
@@ -10709,7 +10711,7 @@
         <x:v>466</x:v>
       </x:c>
       <x:c r="B211" t="s">
-        <x:v>51</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C211">
         <x:v>210</x:v>
@@ -10738,7 +10740,7 @@
         <x:v>466</x:v>
       </x:c>
       <x:c r="B212" t="s">
-        <x:v>51</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C212">
         <x:v>211</x:v>
@@ -10770,7 +10772,7 @@
         <x:v>466</x:v>
       </x:c>
       <x:c r="B213" t="s">
-        <x:v>51</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C213">
         <x:v>212</x:v>
@@ -10805,7 +10807,7 @@
         <x:v>466</x:v>
       </x:c>
       <x:c r="B214" t="s">
-        <x:v>51</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C214">
         <x:v>213</x:v>
@@ -10840,7 +10842,7 @@
         <x:v>466</x:v>
       </x:c>
       <x:c r="B215" t="s">
-        <x:v>51</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C215">
         <x:v>214</x:v>
@@ -10904,7 +10906,7 @@
         <x:v>478</x:v>
       </x:c>
       <x:c r="B217" t="s">
-        <x:v>51</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C217">
         <x:v>216</x:v>
@@ -10916,7 +10918,7 @@
         <x:v>482</x:v>
       </x:c>
       <x:c r="I217" t="str">
-        <x:v>K-</x:v>
+        <x:v>K-40</x:v>
       </x:c>
       <x:c r="L217" t="str">
         <x:v>K-35</x:v>
@@ -10936,7 +10938,7 @@
         <x:v>478</x:v>
       </x:c>
       <x:c r="B218" t="s">
-        <x:v>51</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C218">
         <x:v>217</x:v>
@@ -10974,7 +10976,7 @@
         <x:v>478</x:v>
       </x:c>
       <x:c r="B219" t="s">
-        <x:v>51</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C219">
         <x:v>218</x:v>
@@ -11006,7 +11008,7 @@
         <x:v>478</x:v>
       </x:c>
       <x:c r="B220" t="s">
-        <x:v>51</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C220">
         <x:v>219</x:v>
@@ -11038,7 +11040,7 @@
         <x:v>478</x:v>
       </x:c>
       <x:c r="B221" t="s">
-        <x:v>57</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="C221">
         <x:v>220</x:v>
@@ -11073,7 +11075,7 @@
         <x:v>478</x:v>
       </x:c>
       <x:c r="B222" t="s">
-        <x:v>51</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C222">
         <x:v>221</x:v>
@@ -11102,7 +11104,7 @@
         <x:v>491</x:v>
       </x:c>
       <x:c r="B223" t="s">
-        <x:v>51</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C223">
         <x:v>222</x:v>
@@ -11116,8 +11118,8 @@
       <x:c r="G223" t="s">
         <x:v>493</x:v>
       </x:c>
-      <x:c r="I223" t="s">
-        <x:v>36</x:v>
+      <x:c r="I223" t="str">
+        <x:v>K-46</x:v>
       </x:c>
       <x:c r="L223" t="str">
         <x:v>K-28</x:v>
@@ -11183,8 +11185,8 @@
       <x:c r="G225" t="s">
         <x:v>498</x:v>
       </x:c>
-      <x:c r="I225" t="s">
-        <x:v>36</x:v>
+      <x:c r="I225" t="str">
+        <x:v>K-45</x:v>
       </x:c>
       <x:c r="L225" t="str">
         <x:v>K-29</x:v>
@@ -11218,8 +11220,8 @@
       <x:c r="G226" t="s">
         <x:v>500</x:v>
       </x:c>
-      <x:c r="I226" t="s">
-        <x:v>36</x:v>
+      <x:c r="I226" t="str">
+        <x:v>K-41</x:v>
       </x:c>
       <x:c r="L226" t="str">
         <x:v>K-33</x:v>
@@ -11257,8 +11259,8 @@
       <x:c r="G227" t="s">
         <x:v>502</x:v>
       </x:c>
-      <x:c r="I227" t="s">
-        <x:v>36</x:v>
+      <x:c r="I227" t="str">
+        <x:v>K-43</x:v>
       </x:c>
       <x:c r="L227" t="str">
         <x:v>K-31</x:v>
@@ -11292,8 +11294,8 @@
       <x:c r="G228" t="s">
         <x:v>504</x:v>
       </x:c>
-      <x:c r="I228" t="s">
-        <x:v>36</x:v>
+      <x:c r="I228" t="str">
+        <x:v>K-42</x:v>
       </x:c>
       <x:c r="L228" t="str">
         <x:v>K-32</x:v>
@@ -11370,8 +11372,8 @@
       <x:c r="H230" t="str">
         <x:v>K-39</x:v>
       </x:c>
-      <x:c r="I230" t="s">
-        <x:v>36</x:v>
+      <x:c r="I230" t="str">
+        <x:v>K-44</x:v>
       </x:c>
       <x:c r="K230" t="str">
         <x:v>K-31</x:v>
@@ -11401,7 +11403,7 @@
         <x:v>491</x:v>
       </x:c>
       <x:c r="B231" t="s">
-        <x:v>51</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C231">
         <x:v>230</x:v>
@@ -11434,7 +11436,7 @@
         <x:v>513</x:v>
       </x:c>
       <x:c r="B232" t="s">
-        <x:v>57</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="C232">
         <x:v>231</x:v>
@@ -11448,8 +11450,8 @@
       <x:c r="G232" t="s">
         <x:v>515</x:v>
       </x:c>
-      <x:c r="I232" t="s">
-        <x:v>36</x:v>
+      <x:c r="I232" t="str">
+        <x:v>K-48</x:v>
       </x:c>
       <x:c r="L232" t="str">
         <x:v>K-26</x:v>
@@ -11469,7 +11471,7 @@
         <x:v>513</x:v>
       </x:c>
       <x:c r="B233" t="s">
-        <x:v>51</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C233">
         <x:v>232</x:v>
@@ -11483,8 +11485,8 @@
       <x:c r="G233" t="s">
         <x:v>181</x:v>
       </x:c>
-      <x:c r="I233" t="s">
-        <x:v>36</x:v>
+      <x:c r="I233" t="str">
+        <x:v>K-47</x:v>
       </x:c>
       <x:c r="L233" t="str">
         <x:v>K-27</x:v>
@@ -11506,7 +11508,7 @@
         <x:v>513</x:v>
       </x:c>
       <x:c r="B234" t="s">
-        <x:v>51</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C234">
         <x:v>233</x:v>
@@ -11575,7 +11577,7 @@
         <x:v>513</x:v>
       </x:c>
       <x:c r="B236" t="s">
-        <x:v>53</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="C236">
         <x:v>235</x:v>
@@ -11611,7 +11613,7 @@
         <x:v>513</x:v>
       </x:c>
       <x:c r="B237" t="s">
-        <x:v>53</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="C237">
         <x:v>236</x:v>
@@ -11650,7 +11652,7 @@
         <x:v>513</x:v>
       </x:c>
       <x:c r="B238" t="s">
-        <x:v>53</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="C238">
         <x:v>237</x:v>
@@ -11686,7 +11688,7 @@
         <x:v>513</x:v>
       </x:c>
       <x:c r="B239" t="s">
-        <x:v>53</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="C239">
         <x:v>238</x:v>
@@ -11718,7 +11720,7 @@
         <x:v>513</x:v>
       </x:c>
       <x:c r="B240" t="s">
-        <x:v>51</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C240">
         <x:v>239</x:v>
@@ -11860,7 +11862,7 @@
         <x:v>535</x:v>
       </x:c>
       <x:c r="B244" t="s">
-        <x:v>51</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C244">
         <x:v>243</x:v>
@@ -11871,8 +11873,8 @@
       <x:c r="E244" t="s">
         <x:v>536</x:v>
       </x:c>
-      <x:c r="I244" t="s">
-        <x:v>36</x:v>
+      <x:c r="I244" t="str">
+        <x:v>K-25</x:v>
       </x:c>
       <x:c r="N244"/>
       <x:c r="O244"/>
@@ -11889,7 +11891,7 @@
         <x:v>535</x:v>
       </x:c>
       <x:c r="B245" t="s">
-        <x:v>51</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C245">
         <x:v>244</x:v>
@@ -11903,8 +11905,8 @@
       <x:c r="G245" t="s">
         <x:v>538</x:v>
       </x:c>
-      <x:c r="I245" t="s">
-        <x:v>36</x:v>
+      <x:c r="I245" t="str">
+        <x:v>K-26</x:v>
       </x:c>
       <x:c r="N245"/>
       <x:c r="O245"/>
@@ -11921,7 +11923,7 @@
         <x:v>535</x:v>
       </x:c>
       <x:c r="B246" t="s">
-        <x:v>53</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="C246">
         <x:v>245</x:v>
@@ -11932,8 +11934,8 @@
       <x:c r="E246" t="s">
         <x:v>539</x:v>
       </x:c>
-      <x:c r="I246" t="s">
-        <x:v>36</x:v>
+      <x:c r="I246" t="str">
+        <x:v>K-27</x:v>
       </x:c>
       <x:c r="N246"/>
       <x:c r="O246"/>
@@ -11970,8 +11972,8 @@
       <x:c r="H247" t="s">
         <x:v>96</x:v>
       </x:c>
-      <x:c r="I247" t="s">
-        <x:v>36</x:v>
+      <x:c r="I247" t="str">
+        <x:v>K-24</x:v>
       </x:c>
       <x:c r="J247" t="str">
         <x:v>K-7</x:v>
@@ -12019,8 +12021,8 @@
       <x:c r="E248" t="s">
         <x:v>543</x:v>
       </x:c>
-      <x:c r="I248" t="s">
-        <x:v>36</x:v>
+      <x:c r="I248" t="str">
+        <x:v>K-23</x:v>
       </x:c>
       <x:c r="L248" t="s">
         <x:v>26</x:v>
@@ -12060,8 +12062,8 @@
       <x:c r="H249" t="s">
         <x:v>96</x:v>
       </x:c>
-      <x:c r="I249" t="s">
-        <x:v>36</x:v>
+      <x:c r="I249" t="str">
+        <x:v>K-22</x:v>
       </x:c>
       <x:c r="J249" t="str">
         <x:v>K-6</x:v>
@@ -12098,7 +12100,7 @@
         <x:v>535</x:v>
       </x:c>
       <x:c r="B250" t="s">
-        <x:v>53</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="C250">
         <x:v>249</x:v>
@@ -12127,7 +12129,7 @@
         <x:v>535</x:v>
       </x:c>
       <x:c r="B251" t="s">
-        <x:v>53</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="C251">
         <x:v>250</x:v>
@@ -12161,7 +12163,7 @@
         <x:v>535</x:v>
       </x:c>
       <x:c r="B252" t="s">
-        <x:v>53</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="C252">
         <x:v>251</x:v>
@@ -12195,7 +12197,7 @@
         <x:v>535</x:v>
       </x:c>
       <x:c r="B253" t="s">
-        <x:v>53</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="C253">
         <x:v>252</x:v>
@@ -12209,8 +12211,8 @@
       <x:c r="G253" t="s">
         <x:v>345</x:v>
       </x:c>
-      <x:c r="I253" t="s">
-        <x:v>36</x:v>
+      <x:c r="I253" t="str">
+        <x:v>K-21</x:v>
       </x:c>
       <x:c r="L253" t="s">
         <x:v>26</x:v>
@@ -12234,7 +12236,7 @@
         <x:v>535</x:v>
       </x:c>
       <x:c r="B254" t="s">
-        <x:v>53</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="C254">
         <x:v>253</x:v>
@@ -12263,7 +12265,7 @@
         <x:v>535</x:v>
       </x:c>
       <x:c r="B255" t="s">
-        <x:v>51</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C255">
         <x:v>254</x:v>
@@ -12292,7 +12294,7 @@
         <x:v>535</x:v>
       </x:c>
       <x:c r="B256" t="s">
-        <x:v>51</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C256">
         <x:v>255</x:v>
@@ -12382,7 +12384,7 @@
         <x:v>535</x:v>
       </x:c>
       <x:c r="B259" t="s">
-        <x:v>53</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="C259">
         <x:v>258</x:v>
@@ -12413,7 +12415,7 @@
         <x:v>535</x:v>
       </x:c>
       <x:c r="B260" t="s">
-        <x:v>53</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="C260">
         <x:v>259</x:v>
@@ -12444,7 +12446,7 @@
         <x:v>535</x:v>
       </x:c>
       <x:c r="B261" t="s">
-        <x:v>53</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="C261">
         <x:v>260</x:v>
@@ -12509,7 +12511,7 @@
         <x:v>535</x:v>
       </x:c>
       <x:c r="B263" t="s">
-        <x:v>53</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="C263">
         <x:v>262</x:v>
@@ -12523,9 +12525,7 @@
       <x:c r="H263" t="s">
         <x:v>96</x:v>
       </x:c>
-      <x:c r="J263" t="s">
-        <x:v>36</x:v>
-      </x:c>
+      <x:c r="J263"/>
       <x:c r="K263" t="s">
         <x:v>190</x:v>
       </x:c>
@@ -12546,7 +12546,7 @@
         <x:v>535</x:v>
       </x:c>
       <x:c r="B264" t="s">
-        <x:v>53</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="C264">
         <x:v>263</x:v>
@@ -12557,8 +12557,8 @@
       <x:c r="E264" t="s">
         <x:v>567</x:v>
       </x:c>
-      <x:c r="I264" t="s">
-        <x:v>36</x:v>
+      <x:c r="I264" t="str">
+        <x:v>K-28</x:v>
       </x:c>
       <x:c r="N264"/>
       <x:c r="O264"/>
@@ -12575,7 +12575,7 @@
         <x:v>535</x:v>
       </x:c>
       <x:c r="B265" t="s">
-        <x:v>51</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C265">
         <x:v>264</x:v>
@@ -12617,7 +12617,7 @@
         <x:v>535</x:v>
       </x:c>
       <x:c r="B266" t="s">
-        <x:v>51</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C266">
         <x:v>265</x:v>
@@ -12648,7 +12648,7 @@
         <x:v>535</x:v>
       </x:c>
       <x:c r="B267" t="s">
-        <x:v>51</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C267">
         <x:v>266</x:v>
@@ -12690,7 +12690,7 @@
         <x:v>535</x:v>
       </x:c>
       <x:c r="B268" t="s">
-        <x:v>51</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C268">
         <x:v>267</x:v>
@@ -12728,7 +12728,7 @@
         <x:v>535</x:v>
       </x:c>
       <x:c r="B269" t="s">
-        <x:v>51</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C269">
         <x:v>268</x:v>
@@ -12765,7 +12765,7 @@
         <x:v>535</x:v>
       </x:c>
       <x:c r="B270" t="s">
-        <x:v>57</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="C270">
         <x:v>269</x:v>
@@ -12776,8 +12776,8 @@
       <x:c r="E270" t="s">
         <x:v>577</x:v>
       </x:c>
-      <x:c r="I270" t="s">
-        <x:v>36</x:v>
+      <x:c r="I270" t="str">
+        <x:v>K-33</x:v>
       </x:c>
       <x:c r="L270" t="s">
         <x:v>26</x:v>
@@ -12831,7 +12831,7 @@
         <x:v>535</x:v>
       </x:c>
       <x:c r="B272" t="s">
-        <x:v>51</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C272">
         <x:v>271</x:v>
@@ -12863,7 +12863,7 @@
         <x:v>535</x:v>
       </x:c>
       <x:c r="B273" t="s">
-        <x:v>53</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="C273">
         <x:v>272</x:v>
@@ -12906,8 +12906,8 @@
       <x:c r="H274" t="s">
         <x:v>96</x:v>
       </x:c>
-      <x:c r="I274" t="s">
-        <x:v>36</x:v>
+      <x:c r="I274" t="str">
+        <x:v>K-36</x:v>
       </x:c>
       <x:c r="J274" t="str">
         <x:v>K-15</x:v>
@@ -12942,7 +12942,7 @@
         <x:v>535</x:v>
       </x:c>
       <x:c r="B275" t="s">
-        <x:v>57</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="C275">
         <x:v>274</x:v>
@@ -12957,7 +12957,7 @@
         <x:v>587</x:v>
       </x:c>
       <x:c r="I275" t="str">
-        <x:v>K-</x:v>
+        <x:v>K-13</x:v>
       </x:c>
       <x:c r="L275" t="str">
         <x:v>M-</x:v>
@@ -12995,8 +12995,8 @@
       <x:c r="G276" t="s">
         <x:v>591</x:v>
       </x:c>
-      <x:c r="I276" t="s">
-        <x:v>36</x:v>
+      <x:c r="I276" t="str">
+        <x:v>K-29</x:v>
       </x:c>
       <x:c r="L276" t="s">
         <x:v>26</x:v>
@@ -13059,8 +13059,8 @@
       <x:c r="G278" t="s">
         <x:v>594</x:v>
       </x:c>
-      <x:c r="I278" t="s">
-        <x:v>36</x:v>
+      <x:c r="I278" t="str">
+        <x:v>K-30</x:v>
       </x:c>
       <x:c r="L278" t="s">
         <x:v>26</x:v>
@@ -13084,7 +13084,7 @@
         <x:v>535</x:v>
       </x:c>
       <x:c r="B279" t="s">
-        <x:v>51</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C279">
         <x:v>278</x:v>
@@ -13116,7 +13116,7 @@
         <x:v>535</x:v>
       </x:c>
       <x:c r="B280" t="s">
-        <x:v>53</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="C280">
         <x:v>279</x:v>
@@ -13127,9 +13127,7 @@
       <x:c r="E280" t="s">
         <x:v>598</x:v>
       </x:c>
-      <x:c r="I280" t="s">
-        <x:v>36</x:v>
-      </x:c>
+      <x:c r="I280"/>
       <x:c r="L280" t="s">
         <x:v>26</x:v>
       </x:c>
@@ -13148,7 +13146,7 @@
         <x:v>535</x:v>
       </x:c>
       <x:c r="B281" t="s">
-        <x:v>53</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="C281">
         <x:v>280</x:v>
@@ -13162,9 +13160,7 @@
       <x:c r="G281" t="s">
         <x:v>600</x:v>
       </x:c>
-      <x:c r="I281" t="s">
-        <x:v>36</x:v>
-      </x:c>
+      <x:c r="I281"/>
       <x:c r="L281" t="s">
         <x:v>26</x:v>
       </x:c>
@@ -13183,7 +13179,7 @@
         <x:v>535</x:v>
       </x:c>
       <x:c r="B282" t="s">
-        <x:v>53</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="C282">
         <x:v>281</x:v>
@@ -13197,8 +13193,8 @@
       <x:c r="G282" t="s">
         <x:v>600</x:v>
       </x:c>
-      <x:c r="I282" t="s">
-        <x:v>36</x:v>
+      <x:c r="I282" t="str">
+        <x:v>K-32</x:v>
       </x:c>
       <x:c r="L282" t="s">
         <x:v>26</x:v>
@@ -13220,7 +13216,7 @@
         <x:v>535</x:v>
       </x:c>
       <x:c r="B283" t="s">
-        <x:v>53</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="C283">
         <x:v>282</x:v>
@@ -13234,9 +13230,7 @@
       <x:c r="G283" t="s">
         <x:v>600</x:v>
       </x:c>
-      <x:c r="I283" t="s">
-        <x:v>36</x:v>
-      </x:c>
+      <x:c r="I283"/>
       <x:c r="L283" t="s">
         <x:v>26</x:v>
       </x:c>
@@ -13255,7 +13249,7 @@
         <x:v>535</x:v>
       </x:c>
       <x:c r="B284" t="s">
-        <x:v>53</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="C284">
         <x:v>283</x:v>
@@ -13269,9 +13263,7 @@
       <x:c r="G284" t="s">
         <x:v>604</x:v>
       </x:c>
-      <x:c r="I284" t="s">
-        <x:v>36</x:v>
-      </x:c>
+      <x:c r="I284"/>
       <x:c r="L284" t="s">
         <x:v>26</x:v>
       </x:c>
@@ -13336,8 +13328,8 @@
       <x:c r="G286" t="s">
         <x:v>607</x:v>
       </x:c>
-      <x:c r="I286" t="s">
-        <x:v>36</x:v>
+      <x:c r="I286" t="str">
+        <x:v>K-35</x:v>
       </x:c>
       <x:c r="N286"/>
       <x:c r="O286"/>
@@ -13354,7 +13346,7 @@
         <x:v>535</x:v>
       </x:c>
       <x:c r="B287" t="s">
-        <x:v>51</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C287">
         <x:v>286</x:v>
@@ -13365,8 +13357,8 @@
       <x:c r="E287" t="s">
         <x:v>608</x:v>
       </x:c>
-      <x:c r="I287" t="s">
-        <x:v>36</x:v>
+      <x:c r="I287" t="str">
+        <x:v>K-34</x:v>
       </x:c>
       <x:c r="N287"/>
       <x:c r="O287"/>
@@ -13383,7 +13375,7 @@
         <x:v>535</x:v>
       </x:c>
       <x:c r="B288" t="s">
-        <x:v>53</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="C288">
         <x:v>287</x:v>
@@ -13394,8 +13386,8 @@
       <x:c r="E288" t="s">
         <x:v>609</x:v>
       </x:c>
-      <x:c r="I288" t="s">
-        <x:v>36</x:v>
+      <x:c r="I288" t="str">
+        <x:v>K-31</x:v>
       </x:c>
       <x:c r="L288" t="s">
         <x:v>26</x:v>
@@ -13415,7 +13407,7 @@
         <x:v>610</x:v>
       </x:c>
       <x:c r="B289" t="s">
-        <x:v>51</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C289">
         <x:v>288</x:v>
@@ -13450,7 +13442,7 @@
         <x:v>610</x:v>
       </x:c>
       <x:c r="B290" t="s">
-        <x:v>51</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C290">
         <x:v>289</x:v>
@@ -13517,7 +13509,7 @@
         <x:v>610</x:v>
       </x:c>
       <x:c r="B292" t="s">
-        <x:v>51</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="C292">
         <x:v>291</x:v>
@@ -13631,8 +13623,8 @@
       <x:c r="G295" t="s">
         <x:v>626</x:v>
       </x:c>
-      <x:c r="I295" t="s">
-        <x:v>36</x:v>
+      <x:c r="I295" t="str">
+        <x:v>K-50</x:v>
       </x:c>
       <x:c r="L295" t="str">
         <x:v>K-56</x:v>
@@ -14615,7 +14607,7 @@
         <x:v>21</x:v>
       </x:c>
       <x:c r="B5" t="s">
-        <x:v>54</x:v>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="C5">
         <x:v>1</x:v>
@@ -25998,16 +25990,16 @@
         <x:v>272</x:v>
       </x:c>
       <x:c r="I2" t="s">
-        <x:v>36</x:v>
+        <x:v>62</x:v>
       </x:c>
       <x:c r="J2" t="s">
-        <x:v>36</x:v>
+        <x:v>62</x:v>
       </x:c>
       <x:c r="K2" t="s">
         <x:v>272</x:v>
       </x:c>
       <x:c r="L2" t="s">
-        <x:v>36</x:v>
+        <x:v>62</x:v>
       </x:c>
       <x:c r="M2" t="s">
         <x:v>773</x:v>

</xml_diff>

<commit_message>
Move Saturday paper assignment to Max
</commit_message>
<xml_diff>
--- a/2026年度物件表_KMN置換.xlsx
+++ b/2026年度物件表_KMN置換.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="物件表" sheetId="1" r:id="Rbfabbeee68574edc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日金属（行ってるとこコバ）" sheetId="2" r:id="R45865127cee047e7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日金属収集表  (改定)" sheetId="3" r:id="Rc2f076d1e87b4b0d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日金属収集表  (uejii)" sheetId="4" r:id="R2a70bde4fdc34a5d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日金属収集表 " sheetId="5" r:id="Rfbc4f9ae3eaf40ab"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日可燃収集表 (20250709)" sheetId="6" r:id="Rd77a2ec100b54971"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="土曜日物件表 20250624" sheetId="7" r:id="R01f51ab3c6ce4dce"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ガラ集物件（20250709）" sheetId="8" r:id="R7330d8851b9b413b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="非表示物件" sheetId="9" r:id="R7bbec1230439427a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="土曜日許可物件表（休出用）" sheetId="10" r:id="R55712fdd92114931"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="物件表" sheetId="1" r:id="Rf9b1f7388bec4aa4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日金属（行ってるとこコバ）" sheetId="2" r:id="Rf8597274dd704f1b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日金属収集表  (改定)" sheetId="3" r:id="R263685c45acd4bd8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日金属収集表  (uejii)" sheetId="4" r:id="R97a5f8839ab64a05"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日金属収集表 " sheetId="5" r:id="R543c3443c7f34f73"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日可燃収集表 (20250709)" sheetId="6" r:id="R0ac2467d28e348cb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="土曜日物件表 20250624" sheetId="7" r:id="R08b504c8bed749e2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ガラ集物件（20250709）" sheetId="8" r:id="R8c5b2e7db238484e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="非表示物件" sheetId="9" r:id="R310b803da71c45b7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="土曜日許可物件表（休出用）" sheetId="10" r:id="Re2147025bc33451f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3441,9 +3441,7 @@
       <x:c r="M9" t="str">
         <x:v>段紙</x:v>
       </x:c>
-      <x:c r="N9" t="str">
-        <x:v>段紙(土)-10</x:v>
-      </x:c>
+      <x:c r="N9"/>
       <x:c r="O9"/>
       <x:c r="P9"/>
       <x:c r="Q9"/>
@@ -3484,7 +3482,9 @@
       <x:c r="M10" t="s">
         <x:v>15</x:v>
       </x:c>
-      <x:c r="N10"/>
+      <x:c r="N10" t="str">
+        <x:v>段紙(土)-10</x:v>
+      </x:c>
       <x:c r="O10"/>
       <x:c r="P10"/>
       <x:c r="Q10" t="str">

</xml_diff>

<commit_message>
Update district for property numbers 71 to 74
</commit_message>
<xml_diff>
--- a/2026年度物件表_KMN置換.xlsx
+++ b/2026年度物件表_KMN置換.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="物件表" sheetId="1" r:id="Rf9b1f7388bec4aa4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日金属（行ってるとこコバ）" sheetId="2" r:id="Rf8597274dd704f1b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日金属収集表  (改定)" sheetId="3" r:id="R263685c45acd4bd8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日金属収集表  (uejii)" sheetId="4" r:id="R97a5f8839ab64a05"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日金属収集表 " sheetId="5" r:id="R543c3443c7f34f73"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日可燃収集表 (20250709)" sheetId="6" r:id="R0ac2467d28e348cb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="土曜日物件表 20250624" sheetId="7" r:id="R08b504c8bed749e2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ガラ集物件（20250709）" sheetId="8" r:id="R8c5b2e7db238484e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="非表示物件" sheetId="9" r:id="R310b803da71c45b7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="土曜日許可物件表（休出用）" sheetId="10" r:id="Re2147025bc33451f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="物件表" sheetId="1" r:id="R0e953fae1e524d23"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日金属（行ってるとこコバ）" sheetId="2" r:id="R2c9988d34a084807"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日金属収集表  (改定)" sheetId="3" r:id="R67a226d5569042fe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日金属収集表  (uejii)" sheetId="4" r:id="R8449c3798eff4ab2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日金属収集表 " sheetId="5" r:id="R9c32bc79429342c2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日可燃収集表 (20250709)" sheetId="6" r:id="Rd66261ec94f94368"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="土曜日物件表 20250624" sheetId="7" r:id="Rfcc2d9ecba854b59"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ガラ集物件（20250709）" sheetId="8" r:id="R34494238135d47b9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="非表示物件" sheetId="9" r:id="R1adb1c3642124d0a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="土曜日許可物件表（休出用）" sheetId="10" r:id="R5aaf8a00600f48a4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -5628,8 +5628,8 @@
       <x:c r="V71"/>
     </x:row>
     <x:row r="72" ht="21" customHeight="1">
-      <x:c r="A72" t="s">
-        <x:v>156</x:v>
+      <x:c r="A72" t="str">
+        <x:v>城北</x:v>
       </x:c>
       <x:c r="B72" t="s">
         <x:v>51</x:v>
@@ -5667,8 +5667,8 @@
       <x:c r="V72"/>
     </x:row>
     <x:row r="73" ht="21" customHeight="1">
-      <x:c r="A73" t="s">
-        <x:v>156</x:v>
+      <x:c r="A73" t="str">
+        <x:v>城北</x:v>
       </x:c>
       <x:c r="B73" t="s">
         <x:v>31</x:v>
@@ -5706,8 +5706,8 @@
       </x:c>
     </x:row>
     <x:row r="74" ht="21" customHeight="1">
-      <x:c r="A74" t="s">
-        <x:v>156</x:v>
+      <x:c r="A74" t="str">
+        <x:v>城北</x:v>
       </x:c>
       <x:c r="B74" t="s">
         <x:v>49</x:v>
@@ -5743,8 +5743,8 @@
       </x:c>
     </x:row>
     <x:row r="75" ht="21" customHeight="1">
-      <x:c r="A75" t="s">
-        <x:v>156</x:v>
+      <x:c r="A75" t="str">
+        <x:v>城北</x:v>
       </x:c>
       <x:c r="B75" t="s">
         <x:v>31</x:v>

</xml_diff>

<commit_message>
Apply Friday N collection order update
</commit_message>
<xml_diff>
--- a/2026年度物件表_KMN置換.xlsx
+++ b/2026年度物件表_KMN置換.xlsx
@@ -2,16 +2,16 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="物件表" sheetId="1" r:id="R0e953fae1e524d23"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日金属（行ってるとこコバ）" sheetId="2" r:id="R2c9988d34a084807"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日金属収集表  (改定)" sheetId="3" r:id="R67a226d5569042fe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日金属収集表  (uejii)" sheetId="4" r:id="R8449c3798eff4ab2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日金属収集表 " sheetId="5" r:id="R9c32bc79429342c2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日可燃収集表 (20250709)" sheetId="6" r:id="Rd66261ec94f94368"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="土曜日物件表 20250624" sheetId="7" r:id="Rfcc2d9ecba854b59"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ガラ集物件（20250709）" sheetId="8" r:id="R34494238135d47b9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="非表示物件" sheetId="9" r:id="R1adb1c3642124d0a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="土曜日許可物件表（休出用）" sheetId="10" r:id="R5aaf8a00600f48a4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="物件表" sheetId="1" r:id="Rbbcee19c82ad4183"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日金属（行ってるとこコバ）" sheetId="2" r:id="R46df4e3d21fe4d42"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日金属収集表  (改定)" sheetId="3" r:id="R2b3e4b34cb3e42f8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日金属収集表  (uejii)" sheetId="4" r:id="Rf1990432162a4b76"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日金属収集表 " sheetId="5" r:id="R08d1db8a470f4565"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="水曜日可燃収集表 (20250709)" sheetId="6" r:id="R6186684ba1d0466d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="土曜日物件表 20250624" sheetId="7" r:id="R14c3607202454f7b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ガラ集物件（20250709）" sheetId="8" r:id="R6226204063d946a7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="非表示物件" sheetId="9" r:id="Raeccec5d4eba4044"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="土曜日許可物件表（休出用）" sheetId="10" r:id="R2b4cbf3aa5b64406"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -9062,8 +9062,8 @@
       <x:c r="I163" t="s">
         <x:v>345</x:v>
       </x:c>
-      <x:c r="L163" t="s">
-        <x:v>310</x:v>
+      <x:c r="L163" t="str">
+        <x:v>N-37</x:v>
       </x:c>
       <x:c r="N163"/>
       <x:c r="O163"/>
@@ -9093,8 +9093,8 @@
       <x:c r="E164" t="s">
         <x:v>377</x:v>
       </x:c>
-      <x:c r="L164" t="s">
-        <x:v>305</x:v>
+      <x:c r="L164" t="str">
+        <x:v>N-36</x:v>
       </x:c>
       <x:c r="N164"/>
       <x:c r="O164"/>

</xml_diff>